<commit_message>
Agregar tipo de activo, enlace georreferencial y nivel de criticidad
- Tipo de activo (Poste MT, Suministro, Subestacion) con foto referencial
- Punto georreferencial como enlace de Google Maps (GPS o pegado a mano)
- "Que situacion observa" se reemplaza por "Nivel de criticidad"
  (Riesgo Inminente, Tipo A, B, C) con foto referencial por nivel
- Plantilla Excel, Office Script y payload de ejemplo con campos nuevos
- Guia de Power Automate: nuevo esquema y correo automatico para
  Riesgo Inminente
- Fotos referenciales provisionales (SVG) en img/referencias/

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/power-automate/RegistroPoda_Plantilla.xlsx
+++ b/power-automate/RegistroPoda_Plantilla.xlsx
@@ -146,19 +146,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaPoda" displayName="TablaPoda" ref="A1:J500" headerRowCount="1">
-  <autoFilter ref="A1:J500"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaPoda" displayName="TablaPoda" ref="A1:L500" headerRowCount="1">
+  <autoFilter ref="A1:L500"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Distrito"/>
-    <tableColumn id="3" name="Direccion"/>
-    <tableColumn id="4" name="Latitud"/>
-    <tableColumn id="5" name="Longitud"/>
-    <tableColumn id="6" name="Situacion"/>
-    <tableColumn id="7" name="NombreContacto"/>
-    <tableColumn id="8" name="Telefono"/>
-    <tableColumn id="9" name="EnlacesFotos"/>
-    <tableColumn id="10" name="CarpetaRegistro"/>
+    <tableColumn id="3" name="TipoActivo"/>
+    <tableColumn id="4" name="Direccion"/>
+    <tableColumn id="5" name="UbicacionLink"/>
+    <tableColumn id="6" name="Latitud"/>
+    <tableColumn id="7" name="Longitud"/>
+    <tableColumn id="8" name="Criticidad"/>
+    <tableColumn id="9" name="NombreContacto"/>
+    <tableColumn id="10" name="Telefono"/>
+    <tableColumn id="11" name="EnlacesFotos"/>
+    <tableColumn id="12" name="CarpetaRegistro"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -453,19 +455,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:L500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -481,40 +485,50 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>TipoActivo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Direccion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>UbicacionLink</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Latitud</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Longitud</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Situacion</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Criticidad</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NombreContacto</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Telefono</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>EnlacesFotos</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>CarpetaRegistro</t>
         </is>
@@ -523,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T15:30:00.000Z</t>
+          <t>2026-10-13T15:30:00.000Z</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -533,45 +547,55 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Poste MT</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Av. Los Álamos 123, referencia frente al parque</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=-12.135000,-76.986000</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>-12.135</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>-76.986</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>⚡ Ramas tocando los cables</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Riesgo Inminente</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Juan Pérez</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>987654321</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/SantiagoDeSurco/2026-09/2026-09-17_153000_SantiagoDeSurco/foto1.jpg</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/SantiagoDeSurco/2026-09/2026-09-17_153000_SantiagoDeSurco/</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/Poda/Santiago%20de%20Surco/2026-10/2026-10-13_153000_Santiago%20de%20Surco/foto1.jpg</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/Poda/Santiago%20de%20Surco/2026-10/2026-10-13_153000_Santiago%20de%20Surco/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T09:12:00.000Z</t>
+          <t>2026-10-13T09:12:00.000Z</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -581,34 +605,44 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Subestación</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Jr. Las Begonias 456, cerca al mercado</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>🌳 Árbol caído sobre los cables</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=-12.159000,-76.973000</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>María Torres</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>912345678</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/SanJuanDeMiraflores/2026-09/2026-09-17_091200_SanJuanDeMiraflores/foto1.jpg; https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/SanJuanDeMiraflores/2026-09/2026-09-17_091200_SanJuanDeMiraflores/foto2.jpg</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/SanJuanDeMiraflores/2026-09/2026-09-17_091200_SanJuanDeMiraflores/</t>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/Poda/San%20Juan%20de%20Miraflores/2026-10/2026-10-13_091200_San%20Juan%20de%20Miraflores/foto1.jpg; https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/Poda/San%20Juan%20de%20Miraflores/2026-10/2026-10-13_091200_San%20Juan%20de%20Miraflores/foto2.jpg</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>https://empresa.sharepoint.com/sites/Poda/Documentos%20compartidos/Poda/San%20Juan%20de%20Miraflores/2026-10/2026-10-13_091200_San%20Juan%20de%20Miraflores/</t>
         </is>
       </c>
     </row>
@@ -623,6 +657,8 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -635,6 +671,8 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -647,6 +685,8 @@
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -659,6 +699,8 @@
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -671,6 +713,8 @@
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -683,6 +727,8 @@
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -695,6 +741,8 @@
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -707,6 +755,8 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -719,6 +769,8 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -731,6 +783,8 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -743,6 +797,8 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -755,6 +811,8 @@
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -767,6 +825,8 @@
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -779,6 +839,8 @@
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -791,6 +853,8 @@
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -803,6 +867,8 @@
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -815,6 +881,8 @@
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -827,6 +895,8 @@
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -839,6 +909,8 @@
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -851,6 +923,8 @@
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -863,6 +937,8 @@
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -875,6 +951,8 @@
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -887,6 +965,8 @@
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -899,6 +979,8 @@
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -911,6 +993,8 @@
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -923,6 +1007,8 @@
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -935,6 +1021,8 @@
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -947,6 +1035,8 @@
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -959,6 +1049,8 @@
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -971,6 +1063,8 @@
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
       <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -983,6 +1077,8 @@
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
       <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -995,6 +1091,8 @@
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
       <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -1007,6 +1105,8 @@
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
       <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1019,6 +1119,8 @@
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
       <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -1031,6 +1133,8 @@
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
       <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -1043,6 +1147,8 @@
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
       <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -1055,6 +1161,8 @@
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
       <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1067,6 +1175,8 @@
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="n"/>
       <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1079,6 +1189,8 @@
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="2" t="n"/>
       <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1091,6 +1203,8 @@
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="n"/>
       <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1103,6 +1217,8 @@
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="2" t="n"/>
       <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1115,6 +1231,8 @@
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="n"/>
       <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1127,6 +1245,8 @@
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="n"/>
       <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1139,6 +1259,8 @@
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
       <c r="J47" s="2" t="n"/>
+      <c r="K47" s="2" t="n"/>
+      <c r="L47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1151,6 +1273,8 @@
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
       <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1163,6 +1287,8 @@
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="n"/>
       <c r="J49" s="2" t="n"/>
+      <c r="K49" s="2" t="n"/>
+      <c r="L49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1175,6 +1301,8 @@
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="2" t="n"/>
       <c r="J50" s="2" t="n"/>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1187,6 +1315,8 @@
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
       <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1199,6 +1329,8 @@
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
       <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1211,6 +1343,8 @@
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1223,6 +1357,8 @@
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
       <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1235,6 +1371,8 @@
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
       <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1247,6 +1385,8 @@
       <c r="H56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
       <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1259,6 +1399,8 @@
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
       <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1271,6 +1413,8 @@
       <c r="H58" s="2" t="n"/>
       <c r="I58" s="2" t="n"/>
       <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1283,6 +1427,8 @@
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
       <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1295,6 +1441,8 @@
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
       <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1307,6 +1455,8 @@
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="n"/>
       <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1319,6 +1469,8 @@
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="n"/>
       <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1331,6 +1483,8 @@
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="n"/>
       <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1343,6 +1497,8 @@
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="n"/>
       <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1355,6 +1511,8 @@
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="n"/>
       <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1367,6 +1525,8 @@
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="n"/>
       <c r="J66" s="2" t="n"/>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1379,6 +1539,8 @@
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1391,6 +1553,8 @@
       <c r="H68" s="2" t="n"/>
       <c r="I68" s="2" t="n"/>
       <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1403,6 +1567,8 @@
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1415,6 +1581,8 @@
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="n"/>
       <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1427,6 +1595,8 @@
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="2" t="n"/>
       <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1439,6 +1609,8 @@
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="n"/>
       <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1451,6 +1623,8 @@
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="2" t="n"/>
       <c r="J73" s="2" t="n"/>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1463,6 +1637,8 @@
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="2" t="n"/>
+      <c r="K74" s="2" t="n"/>
+      <c r="L74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1475,6 +1651,8 @@
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="n"/>
       <c r="J75" s="2" t="n"/>
+      <c r="K75" s="2" t="n"/>
+      <c r="L75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1487,6 +1665,8 @@
       <c r="H76" s="2" t="n"/>
       <c r="I76" s="2" t="n"/>
       <c r="J76" s="2" t="n"/>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1499,6 +1679,8 @@
       <c r="H77" s="2" t="n"/>
       <c r="I77" s="2" t="n"/>
       <c r="J77" s="2" t="n"/>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1511,6 +1693,8 @@
       <c r="H78" s="2" t="n"/>
       <c r="I78" s="2" t="n"/>
       <c r="J78" s="2" t="n"/>
+      <c r="K78" s="2" t="n"/>
+      <c r="L78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1523,6 +1707,8 @@
       <c r="H79" s="2" t="n"/>
       <c r="I79" s="2" t="n"/>
       <c r="J79" s="2" t="n"/>
+      <c r="K79" s="2" t="n"/>
+      <c r="L79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1535,6 +1721,8 @@
       <c r="H80" s="2" t="n"/>
       <c r="I80" s="2" t="n"/>
       <c r="J80" s="2" t="n"/>
+      <c r="K80" s="2" t="n"/>
+      <c r="L80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1547,6 +1735,8 @@
       <c r="H81" s="2" t="n"/>
       <c r="I81" s="2" t="n"/>
       <c r="J81" s="2" t="n"/>
+      <c r="K81" s="2" t="n"/>
+      <c r="L81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1559,6 +1749,8 @@
       <c r="H82" s="2" t="n"/>
       <c r="I82" s="2" t="n"/>
       <c r="J82" s="2" t="n"/>
+      <c r="K82" s="2" t="n"/>
+      <c r="L82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1571,6 +1763,8 @@
       <c r="H83" s="2" t="n"/>
       <c r="I83" s="2" t="n"/>
       <c r="J83" s="2" t="n"/>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1583,6 +1777,8 @@
       <c r="H84" s="2" t="n"/>
       <c r="I84" s="2" t="n"/>
       <c r="J84" s="2" t="n"/>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1595,6 +1791,8 @@
       <c r="H85" s="2" t="n"/>
       <c r="I85" s="2" t="n"/>
       <c r="J85" s="2" t="n"/>
+      <c r="K85" s="2" t="n"/>
+      <c r="L85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1607,6 +1805,8 @@
       <c r="H86" s="2" t="n"/>
       <c r="I86" s="2" t="n"/>
       <c r="J86" s="2" t="n"/>
+      <c r="K86" s="2" t="n"/>
+      <c r="L86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1619,6 +1819,8 @@
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="n"/>
       <c r="J87" s="2" t="n"/>
+      <c r="K87" s="2" t="n"/>
+      <c r="L87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1631,6 +1833,8 @@
       <c r="H88" s="2" t="n"/>
       <c r="I88" s="2" t="n"/>
       <c r="J88" s="2" t="n"/>
+      <c r="K88" s="2" t="n"/>
+      <c r="L88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1643,6 +1847,8 @@
       <c r="H89" s="2" t="n"/>
       <c r="I89" s="2" t="n"/>
       <c r="J89" s="2" t="n"/>
+      <c r="K89" s="2" t="n"/>
+      <c r="L89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1655,6 +1861,8 @@
       <c r="H90" s="2" t="n"/>
       <c r="I90" s="2" t="n"/>
       <c r="J90" s="2" t="n"/>
+      <c r="K90" s="2" t="n"/>
+      <c r="L90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1667,6 +1875,8 @@
       <c r="H91" s="2" t="n"/>
       <c r="I91" s="2" t="n"/>
       <c r="J91" s="2" t="n"/>
+      <c r="K91" s="2" t="n"/>
+      <c r="L91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1679,6 +1889,8 @@
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="2" t="n"/>
       <c r="J92" s="2" t="n"/>
+      <c r="K92" s="2" t="n"/>
+      <c r="L92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1691,6 +1903,8 @@
       <c r="H93" s="2" t="n"/>
       <c r="I93" s="2" t="n"/>
       <c r="J93" s="2" t="n"/>
+      <c r="K93" s="2" t="n"/>
+      <c r="L93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1703,6 +1917,8 @@
       <c r="H94" s="2" t="n"/>
       <c r="I94" s="2" t="n"/>
       <c r="J94" s="2" t="n"/>
+      <c r="K94" s="2" t="n"/>
+      <c r="L94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -1715,6 +1931,8 @@
       <c r="H95" s="2" t="n"/>
       <c r="I95" s="2" t="n"/>
       <c r="J95" s="2" t="n"/>
+      <c r="K95" s="2" t="n"/>
+      <c r="L95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -1727,6 +1945,8 @@
       <c r="H96" s="2" t="n"/>
       <c r="I96" s="2" t="n"/>
       <c r="J96" s="2" t="n"/>
+      <c r="K96" s="2" t="n"/>
+      <c r="L96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -1739,6 +1959,8 @@
       <c r="H97" s="2" t="n"/>
       <c r="I97" s="2" t="n"/>
       <c r="J97" s="2" t="n"/>
+      <c r="K97" s="2" t="n"/>
+      <c r="L97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -1751,6 +1973,8 @@
       <c r="H98" s="2" t="n"/>
       <c r="I98" s="2" t="n"/>
       <c r="J98" s="2" t="n"/>
+      <c r="K98" s="2" t="n"/>
+      <c r="L98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -1763,6 +1987,8 @@
       <c r="H99" s="2" t="n"/>
       <c r="I99" s="2" t="n"/>
       <c r="J99" s="2" t="n"/>
+      <c r="K99" s="2" t="n"/>
+      <c r="L99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -1775,6 +2001,8 @@
       <c r="H100" s="2" t="n"/>
       <c r="I100" s="2" t="n"/>
       <c r="J100" s="2" t="n"/>
+      <c r="K100" s="2" t="n"/>
+      <c r="L100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -1787,6 +2015,8 @@
       <c r="H101" s="2" t="n"/>
       <c r="I101" s="2" t="n"/>
       <c r="J101" s="2" t="n"/>
+      <c r="K101" s="2" t="n"/>
+      <c r="L101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -1799,6 +2029,8 @@
       <c r="H102" s="2" t="n"/>
       <c r="I102" s="2" t="n"/>
       <c r="J102" s="2" t="n"/>
+      <c r="K102" s="2" t="n"/>
+      <c r="L102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -1811,6 +2043,8 @@
       <c r="H103" s="2" t="n"/>
       <c r="I103" s="2" t="n"/>
       <c r="J103" s="2" t="n"/>
+      <c r="K103" s="2" t="n"/>
+      <c r="L103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -1823,6 +2057,8 @@
       <c r="H104" s="2" t="n"/>
       <c r="I104" s="2" t="n"/>
       <c r="J104" s="2" t="n"/>
+      <c r="K104" s="2" t="n"/>
+      <c r="L104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -1835,6 +2071,8 @@
       <c r="H105" s="2" t="n"/>
       <c r="I105" s="2" t="n"/>
       <c r="J105" s="2" t="n"/>
+      <c r="K105" s="2" t="n"/>
+      <c r="L105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -1847,6 +2085,8 @@
       <c r="H106" s="2" t="n"/>
       <c r="I106" s="2" t="n"/>
       <c r="J106" s="2" t="n"/>
+      <c r="K106" s="2" t="n"/>
+      <c r="L106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -1859,6 +2099,8 @@
       <c r="H107" s="2" t="n"/>
       <c r="I107" s="2" t="n"/>
       <c r="J107" s="2" t="n"/>
+      <c r="K107" s="2" t="n"/>
+      <c r="L107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -1871,6 +2113,8 @@
       <c r="H108" s="2" t="n"/>
       <c r="I108" s="2" t="n"/>
       <c r="J108" s="2" t="n"/>
+      <c r="K108" s="2" t="n"/>
+      <c r="L108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -1883,6 +2127,8 @@
       <c r="H109" s="2" t="n"/>
       <c r="I109" s="2" t="n"/>
       <c r="J109" s="2" t="n"/>
+      <c r="K109" s="2" t="n"/>
+      <c r="L109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -1895,6 +2141,8 @@
       <c r="H110" s="2" t="n"/>
       <c r="I110" s="2" t="n"/>
       <c r="J110" s="2" t="n"/>
+      <c r="K110" s="2" t="n"/>
+      <c r="L110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -1907,6 +2155,8 @@
       <c r="H111" s="2" t="n"/>
       <c r="I111" s="2" t="n"/>
       <c r="J111" s="2" t="n"/>
+      <c r="K111" s="2" t="n"/>
+      <c r="L111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -1919,6 +2169,8 @@
       <c r="H112" s="2" t="n"/>
       <c r="I112" s="2" t="n"/>
       <c r="J112" s="2" t="n"/>
+      <c r="K112" s="2" t="n"/>
+      <c r="L112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -1931,6 +2183,8 @@
       <c r="H113" s="2" t="n"/>
       <c r="I113" s="2" t="n"/>
       <c r="J113" s="2" t="n"/>
+      <c r="K113" s="2" t="n"/>
+      <c r="L113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -1943,6 +2197,8 @@
       <c r="H114" s="2" t="n"/>
       <c r="I114" s="2" t="n"/>
       <c r="J114" s="2" t="n"/>
+      <c r="K114" s="2" t="n"/>
+      <c r="L114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -1955,6 +2211,8 @@
       <c r="H115" s="2" t="n"/>
       <c r="I115" s="2" t="n"/>
       <c r="J115" s="2" t="n"/>
+      <c r="K115" s="2" t="n"/>
+      <c r="L115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -1967,6 +2225,8 @@
       <c r="H116" s="2" t="n"/>
       <c r="I116" s="2" t="n"/>
       <c r="J116" s="2" t="n"/>
+      <c r="K116" s="2" t="n"/>
+      <c r="L116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -1979,6 +2239,8 @@
       <c r="H117" s="2" t="n"/>
       <c r="I117" s="2" t="n"/>
       <c r="J117" s="2" t="n"/>
+      <c r="K117" s="2" t="n"/>
+      <c r="L117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -1991,6 +2253,8 @@
       <c r="H118" s="2" t="n"/>
       <c r="I118" s="2" t="n"/>
       <c r="J118" s="2" t="n"/>
+      <c r="K118" s="2" t="n"/>
+      <c r="L118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -2003,6 +2267,8 @@
       <c r="H119" s="2" t="n"/>
       <c r="I119" s="2" t="n"/>
       <c r="J119" s="2" t="n"/>
+      <c r="K119" s="2" t="n"/>
+      <c r="L119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -2015,6 +2281,8 @@
       <c r="H120" s="2" t="n"/>
       <c r="I120" s="2" t="n"/>
       <c r="J120" s="2" t="n"/>
+      <c r="K120" s="2" t="n"/>
+      <c r="L120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -2027,6 +2295,8 @@
       <c r="H121" s="2" t="n"/>
       <c r="I121" s="2" t="n"/>
       <c r="J121" s="2" t="n"/>
+      <c r="K121" s="2" t="n"/>
+      <c r="L121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -2039,6 +2309,8 @@
       <c r="H122" s="2" t="n"/>
       <c r="I122" s="2" t="n"/>
       <c r="J122" s="2" t="n"/>
+      <c r="K122" s="2" t="n"/>
+      <c r="L122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -2051,6 +2323,8 @@
       <c r="H123" s="2" t="n"/>
       <c r="I123" s="2" t="n"/>
       <c r="J123" s="2" t="n"/>
+      <c r="K123" s="2" t="n"/>
+      <c r="L123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -2063,6 +2337,8 @@
       <c r="H124" s="2" t="n"/>
       <c r="I124" s="2" t="n"/>
       <c r="J124" s="2" t="n"/>
+      <c r="K124" s="2" t="n"/>
+      <c r="L124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -2075,6 +2351,8 @@
       <c r="H125" s="2" t="n"/>
       <c r="I125" s="2" t="n"/>
       <c r="J125" s="2" t="n"/>
+      <c r="K125" s="2" t="n"/>
+      <c r="L125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -2087,6 +2365,8 @@
       <c r="H126" s="2" t="n"/>
       <c r="I126" s="2" t="n"/>
       <c r="J126" s="2" t="n"/>
+      <c r="K126" s="2" t="n"/>
+      <c r="L126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -2099,6 +2379,8 @@
       <c r="H127" s="2" t="n"/>
       <c r="I127" s="2" t="n"/>
       <c r="J127" s="2" t="n"/>
+      <c r="K127" s="2" t="n"/>
+      <c r="L127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -2111,6 +2393,8 @@
       <c r="H128" s="2" t="n"/>
       <c r="I128" s="2" t="n"/>
       <c r="J128" s="2" t="n"/>
+      <c r="K128" s="2" t="n"/>
+      <c r="L128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -2123,6 +2407,8 @@
       <c r="H129" s="2" t="n"/>
       <c r="I129" s="2" t="n"/>
       <c r="J129" s="2" t="n"/>
+      <c r="K129" s="2" t="n"/>
+      <c r="L129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -2135,6 +2421,8 @@
       <c r="H130" s="2" t="n"/>
       <c r="I130" s="2" t="n"/>
       <c r="J130" s="2" t="n"/>
+      <c r="K130" s="2" t="n"/>
+      <c r="L130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -2147,6 +2435,8 @@
       <c r="H131" s="2" t="n"/>
       <c r="I131" s="2" t="n"/>
       <c r="J131" s="2" t="n"/>
+      <c r="K131" s="2" t="n"/>
+      <c r="L131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -2159,6 +2449,8 @@
       <c r="H132" s="2" t="n"/>
       <c r="I132" s="2" t="n"/>
       <c r="J132" s="2" t="n"/>
+      <c r="K132" s="2" t="n"/>
+      <c r="L132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -2171,6 +2463,8 @@
       <c r="H133" s="2" t="n"/>
       <c r="I133" s="2" t="n"/>
       <c r="J133" s="2" t="n"/>
+      <c r="K133" s="2" t="n"/>
+      <c r="L133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -2183,6 +2477,8 @@
       <c r="H134" s="2" t="n"/>
       <c r="I134" s="2" t="n"/>
       <c r="J134" s="2" t="n"/>
+      <c r="K134" s="2" t="n"/>
+      <c r="L134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -2195,6 +2491,8 @@
       <c r="H135" s="2" t="n"/>
       <c r="I135" s="2" t="n"/>
       <c r="J135" s="2" t="n"/>
+      <c r="K135" s="2" t="n"/>
+      <c r="L135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -2207,6 +2505,8 @@
       <c r="H136" s="2" t="n"/>
       <c r="I136" s="2" t="n"/>
       <c r="J136" s="2" t="n"/>
+      <c r="K136" s="2" t="n"/>
+      <c r="L136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -2219,6 +2519,8 @@
       <c r="H137" s="2" t="n"/>
       <c r="I137" s="2" t="n"/>
       <c r="J137" s="2" t="n"/>
+      <c r="K137" s="2" t="n"/>
+      <c r="L137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -2231,6 +2533,8 @@
       <c r="H138" s="2" t="n"/>
       <c r="I138" s="2" t="n"/>
       <c r="J138" s="2" t="n"/>
+      <c r="K138" s="2" t="n"/>
+      <c r="L138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -2243,6 +2547,8 @@
       <c r="H139" s="2" t="n"/>
       <c r="I139" s="2" t="n"/>
       <c r="J139" s="2" t="n"/>
+      <c r="K139" s="2" t="n"/>
+      <c r="L139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -2255,6 +2561,8 @@
       <c r="H140" s="2" t="n"/>
       <c r="I140" s="2" t="n"/>
       <c r="J140" s="2" t="n"/>
+      <c r="K140" s="2" t="n"/>
+      <c r="L140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -2267,6 +2575,8 @@
       <c r="H141" s="2" t="n"/>
       <c r="I141" s="2" t="n"/>
       <c r="J141" s="2" t="n"/>
+      <c r="K141" s="2" t="n"/>
+      <c r="L141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -2279,6 +2589,8 @@
       <c r="H142" s="2" t="n"/>
       <c r="I142" s="2" t="n"/>
       <c r="J142" s="2" t="n"/>
+      <c r="K142" s="2" t="n"/>
+      <c r="L142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -2291,6 +2603,8 @@
       <c r="H143" s="2" t="n"/>
       <c r="I143" s="2" t="n"/>
       <c r="J143" s="2" t="n"/>
+      <c r="K143" s="2" t="n"/>
+      <c r="L143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -2303,6 +2617,8 @@
       <c r="H144" s="2" t="n"/>
       <c r="I144" s="2" t="n"/>
       <c r="J144" s="2" t="n"/>
+      <c r="K144" s="2" t="n"/>
+      <c r="L144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -2315,6 +2631,8 @@
       <c r="H145" s="2" t="n"/>
       <c r="I145" s="2" t="n"/>
       <c r="J145" s="2" t="n"/>
+      <c r="K145" s="2" t="n"/>
+      <c r="L145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -2327,6 +2645,8 @@
       <c r="H146" s="2" t="n"/>
       <c r="I146" s="2" t="n"/>
       <c r="J146" s="2" t="n"/>
+      <c r="K146" s="2" t="n"/>
+      <c r="L146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -2339,6 +2659,8 @@
       <c r="H147" s="2" t="n"/>
       <c r="I147" s="2" t="n"/>
       <c r="J147" s="2" t="n"/>
+      <c r="K147" s="2" t="n"/>
+      <c r="L147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -2351,6 +2673,8 @@
       <c r="H148" s="2" t="n"/>
       <c r="I148" s="2" t="n"/>
       <c r="J148" s="2" t="n"/>
+      <c r="K148" s="2" t="n"/>
+      <c r="L148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -2363,6 +2687,8 @@
       <c r="H149" s="2" t="n"/>
       <c r="I149" s="2" t="n"/>
       <c r="J149" s="2" t="n"/>
+      <c r="K149" s="2" t="n"/>
+      <c r="L149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -2375,6 +2701,8 @@
       <c r="H150" s="2" t="n"/>
       <c r="I150" s="2" t="n"/>
       <c r="J150" s="2" t="n"/>
+      <c r="K150" s="2" t="n"/>
+      <c r="L150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -2387,6 +2715,8 @@
       <c r="H151" s="2" t="n"/>
       <c r="I151" s="2" t="n"/>
       <c r="J151" s="2" t="n"/>
+      <c r="K151" s="2" t="n"/>
+      <c r="L151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -2399,6 +2729,8 @@
       <c r="H152" s="2" t="n"/>
       <c r="I152" s="2" t="n"/>
       <c r="J152" s="2" t="n"/>
+      <c r="K152" s="2" t="n"/>
+      <c r="L152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -2411,6 +2743,8 @@
       <c r="H153" s="2" t="n"/>
       <c r="I153" s="2" t="n"/>
       <c r="J153" s="2" t="n"/>
+      <c r="K153" s="2" t="n"/>
+      <c r="L153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -2423,6 +2757,8 @@
       <c r="H154" s="2" t="n"/>
       <c r="I154" s="2" t="n"/>
       <c r="J154" s="2" t="n"/>
+      <c r="K154" s="2" t="n"/>
+      <c r="L154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -2435,6 +2771,8 @@
       <c r="H155" s="2" t="n"/>
       <c r="I155" s="2" t="n"/>
       <c r="J155" s="2" t="n"/>
+      <c r="K155" s="2" t="n"/>
+      <c r="L155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -2447,6 +2785,8 @@
       <c r="H156" s="2" t="n"/>
       <c r="I156" s="2" t="n"/>
       <c r="J156" s="2" t="n"/>
+      <c r="K156" s="2" t="n"/>
+      <c r="L156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -2459,6 +2799,8 @@
       <c r="H157" s="2" t="n"/>
       <c r="I157" s="2" t="n"/>
       <c r="J157" s="2" t="n"/>
+      <c r="K157" s="2" t="n"/>
+      <c r="L157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -2471,6 +2813,8 @@
       <c r="H158" s="2" t="n"/>
       <c r="I158" s="2" t="n"/>
       <c r="J158" s="2" t="n"/>
+      <c r="K158" s="2" t="n"/>
+      <c r="L158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -2483,6 +2827,8 @@
       <c r="H159" s="2" t="n"/>
       <c r="I159" s="2" t="n"/>
       <c r="J159" s="2" t="n"/>
+      <c r="K159" s="2" t="n"/>
+      <c r="L159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -2495,6 +2841,8 @@
       <c r="H160" s="2" t="n"/>
       <c r="I160" s="2" t="n"/>
       <c r="J160" s="2" t="n"/>
+      <c r="K160" s="2" t="n"/>
+      <c r="L160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -2507,6 +2855,8 @@
       <c r="H161" s="2" t="n"/>
       <c r="I161" s="2" t="n"/>
       <c r="J161" s="2" t="n"/>
+      <c r="K161" s="2" t="n"/>
+      <c r="L161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -2519,6 +2869,8 @@
       <c r="H162" s="2" t="n"/>
       <c r="I162" s="2" t="n"/>
       <c r="J162" s="2" t="n"/>
+      <c r="K162" s="2" t="n"/>
+      <c r="L162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -2531,6 +2883,8 @@
       <c r="H163" s="2" t="n"/>
       <c r="I163" s="2" t="n"/>
       <c r="J163" s="2" t="n"/>
+      <c r="K163" s="2" t="n"/>
+      <c r="L163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -2543,6 +2897,8 @@
       <c r="H164" s="2" t="n"/>
       <c r="I164" s="2" t="n"/>
       <c r="J164" s="2" t="n"/>
+      <c r="K164" s="2" t="n"/>
+      <c r="L164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -2555,6 +2911,8 @@
       <c r="H165" s="2" t="n"/>
       <c r="I165" s="2" t="n"/>
       <c r="J165" s="2" t="n"/>
+      <c r="K165" s="2" t="n"/>
+      <c r="L165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -2567,6 +2925,8 @@
       <c r="H166" s="2" t="n"/>
       <c r="I166" s="2" t="n"/>
       <c r="J166" s="2" t="n"/>
+      <c r="K166" s="2" t="n"/>
+      <c r="L166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -2579,6 +2939,8 @@
       <c r="H167" s="2" t="n"/>
       <c r="I167" s="2" t="n"/>
       <c r="J167" s="2" t="n"/>
+      <c r="K167" s="2" t="n"/>
+      <c r="L167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -2591,6 +2953,8 @@
       <c r="H168" s="2" t="n"/>
       <c r="I168" s="2" t="n"/>
       <c r="J168" s="2" t="n"/>
+      <c r="K168" s="2" t="n"/>
+      <c r="L168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -2603,6 +2967,8 @@
       <c r="H169" s="2" t="n"/>
       <c r="I169" s="2" t="n"/>
       <c r="J169" s="2" t="n"/>
+      <c r="K169" s="2" t="n"/>
+      <c r="L169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -2615,6 +2981,8 @@
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="n"/>
       <c r="J170" s="2" t="n"/>
+      <c r="K170" s="2" t="n"/>
+      <c r="L170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -2627,6 +2995,8 @@
       <c r="H171" s="2" t="n"/>
       <c r="I171" s="2" t="n"/>
       <c r="J171" s="2" t="n"/>
+      <c r="K171" s="2" t="n"/>
+      <c r="L171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -2639,6 +3009,8 @@
       <c r="H172" s="2" t="n"/>
       <c r="I172" s="2" t="n"/>
       <c r="J172" s="2" t="n"/>
+      <c r="K172" s="2" t="n"/>
+      <c r="L172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -2651,6 +3023,8 @@
       <c r="H173" s="2" t="n"/>
       <c r="I173" s="2" t="n"/>
       <c r="J173" s="2" t="n"/>
+      <c r="K173" s="2" t="n"/>
+      <c r="L173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -2663,6 +3037,8 @@
       <c r="H174" s="2" t="n"/>
       <c r="I174" s="2" t="n"/>
       <c r="J174" s="2" t="n"/>
+      <c r="K174" s="2" t="n"/>
+      <c r="L174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -2675,6 +3051,8 @@
       <c r="H175" s="2" t="n"/>
       <c r="I175" s="2" t="n"/>
       <c r="J175" s="2" t="n"/>
+      <c r="K175" s="2" t="n"/>
+      <c r="L175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -2687,6 +3065,8 @@
       <c r="H176" s="2" t="n"/>
       <c r="I176" s="2" t="n"/>
       <c r="J176" s="2" t="n"/>
+      <c r="K176" s="2" t="n"/>
+      <c r="L176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -2699,6 +3079,8 @@
       <c r="H177" s="2" t="n"/>
       <c r="I177" s="2" t="n"/>
       <c r="J177" s="2" t="n"/>
+      <c r="K177" s="2" t="n"/>
+      <c r="L177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -2711,6 +3093,8 @@
       <c r="H178" s="2" t="n"/>
       <c r="I178" s="2" t="n"/>
       <c r="J178" s="2" t="n"/>
+      <c r="K178" s="2" t="n"/>
+      <c r="L178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -2723,6 +3107,8 @@
       <c r="H179" s="2" t="n"/>
       <c r="I179" s="2" t="n"/>
       <c r="J179" s="2" t="n"/>
+      <c r="K179" s="2" t="n"/>
+      <c r="L179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -2735,6 +3121,8 @@
       <c r="H180" s="2" t="n"/>
       <c r="I180" s="2" t="n"/>
       <c r="J180" s="2" t="n"/>
+      <c r="K180" s="2" t="n"/>
+      <c r="L180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -2747,6 +3135,8 @@
       <c r="H181" s="2" t="n"/>
       <c r="I181" s="2" t="n"/>
       <c r="J181" s="2" t="n"/>
+      <c r="K181" s="2" t="n"/>
+      <c r="L181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -2759,6 +3149,8 @@
       <c r="H182" s="2" t="n"/>
       <c r="I182" s="2" t="n"/>
       <c r="J182" s="2" t="n"/>
+      <c r="K182" s="2" t="n"/>
+      <c r="L182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -2771,6 +3163,8 @@
       <c r="H183" s="2" t="n"/>
       <c r="I183" s="2" t="n"/>
       <c r="J183" s="2" t="n"/>
+      <c r="K183" s="2" t="n"/>
+      <c r="L183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -2783,6 +3177,8 @@
       <c r="H184" s="2" t="n"/>
       <c r="I184" s="2" t="n"/>
       <c r="J184" s="2" t="n"/>
+      <c r="K184" s="2" t="n"/>
+      <c r="L184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -2795,6 +3191,8 @@
       <c r="H185" s="2" t="n"/>
       <c r="I185" s="2" t="n"/>
       <c r="J185" s="2" t="n"/>
+      <c r="K185" s="2" t="n"/>
+      <c r="L185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -2807,6 +3205,8 @@
       <c r="H186" s="2" t="n"/>
       <c r="I186" s="2" t="n"/>
       <c r="J186" s="2" t="n"/>
+      <c r="K186" s="2" t="n"/>
+      <c r="L186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -2819,6 +3219,8 @@
       <c r="H187" s="2" t="n"/>
       <c r="I187" s="2" t="n"/>
       <c r="J187" s="2" t="n"/>
+      <c r="K187" s="2" t="n"/>
+      <c r="L187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -2831,6 +3233,8 @@
       <c r="H188" s="2" t="n"/>
       <c r="I188" s="2" t="n"/>
       <c r="J188" s="2" t="n"/>
+      <c r="K188" s="2" t="n"/>
+      <c r="L188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -2843,6 +3247,8 @@
       <c r="H189" s="2" t="n"/>
       <c r="I189" s="2" t="n"/>
       <c r="J189" s="2" t="n"/>
+      <c r="K189" s="2" t="n"/>
+      <c r="L189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -2855,6 +3261,8 @@
       <c r="H190" s="2" t="n"/>
       <c r="I190" s="2" t="n"/>
       <c r="J190" s="2" t="n"/>
+      <c r="K190" s="2" t="n"/>
+      <c r="L190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -2867,6 +3275,8 @@
       <c r="H191" s="2" t="n"/>
       <c r="I191" s="2" t="n"/>
       <c r="J191" s="2" t="n"/>
+      <c r="K191" s="2" t="n"/>
+      <c r="L191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -2879,6 +3289,8 @@
       <c r="H192" s="2" t="n"/>
       <c r="I192" s="2" t="n"/>
       <c r="J192" s="2" t="n"/>
+      <c r="K192" s="2" t="n"/>
+      <c r="L192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -2891,6 +3303,8 @@
       <c r="H193" s="2" t="n"/>
       <c r="I193" s="2" t="n"/>
       <c r="J193" s="2" t="n"/>
+      <c r="K193" s="2" t="n"/>
+      <c r="L193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -2903,6 +3317,8 @@
       <c r="H194" s="2" t="n"/>
       <c r="I194" s="2" t="n"/>
       <c r="J194" s="2" t="n"/>
+      <c r="K194" s="2" t="n"/>
+      <c r="L194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -2915,6 +3331,8 @@
       <c r="H195" s="2" t="n"/>
       <c r="I195" s="2" t="n"/>
       <c r="J195" s="2" t="n"/>
+      <c r="K195" s="2" t="n"/>
+      <c r="L195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -2927,6 +3345,8 @@
       <c r="H196" s="2" t="n"/>
       <c r="I196" s="2" t="n"/>
       <c r="J196" s="2" t="n"/>
+      <c r="K196" s="2" t="n"/>
+      <c r="L196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -2939,6 +3359,8 @@
       <c r="H197" s="2" t="n"/>
       <c r="I197" s="2" t="n"/>
       <c r="J197" s="2" t="n"/>
+      <c r="K197" s="2" t="n"/>
+      <c r="L197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -2951,6 +3373,8 @@
       <c r="H198" s="2" t="n"/>
       <c r="I198" s="2" t="n"/>
       <c r="J198" s="2" t="n"/>
+      <c r="K198" s="2" t="n"/>
+      <c r="L198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -2963,6 +3387,8 @@
       <c r="H199" s="2" t="n"/>
       <c r="I199" s="2" t="n"/>
       <c r="J199" s="2" t="n"/>
+      <c r="K199" s="2" t="n"/>
+      <c r="L199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -2975,6 +3401,8 @@
       <c r="H200" s="2" t="n"/>
       <c r="I200" s="2" t="n"/>
       <c r="J200" s="2" t="n"/>
+      <c r="K200" s="2" t="n"/>
+      <c r="L200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
@@ -2987,6 +3415,8 @@
       <c r="H201" s="2" t="n"/>
       <c r="I201" s="2" t="n"/>
       <c r="J201" s="2" t="n"/>
+      <c r="K201" s="2" t="n"/>
+      <c r="L201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n"/>
@@ -2999,6 +3429,8 @@
       <c r="H202" s="2" t="n"/>
       <c r="I202" s="2" t="n"/>
       <c r="J202" s="2" t="n"/>
+      <c r="K202" s="2" t="n"/>
+      <c r="L202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n"/>
@@ -3011,6 +3443,8 @@
       <c r="H203" s="2" t="n"/>
       <c r="I203" s="2" t="n"/>
       <c r="J203" s="2" t="n"/>
+      <c r="K203" s="2" t="n"/>
+      <c r="L203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n"/>
@@ -3023,6 +3457,8 @@
       <c r="H204" s="2" t="n"/>
       <c r="I204" s="2" t="n"/>
       <c r="J204" s="2" t="n"/>
+      <c r="K204" s="2" t="n"/>
+      <c r="L204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
@@ -3035,6 +3471,8 @@
       <c r="H205" s="2" t="n"/>
       <c r="I205" s="2" t="n"/>
       <c r="J205" s="2" t="n"/>
+      <c r="K205" s="2" t="n"/>
+      <c r="L205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n"/>
@@ -3047,6 +3485,8 @@
       <c r="H206" s="2" t="n"/>
       <c r="I206" s="2" t="n"/>
       <c r="J206" s="2" t="n"/>
+      <c r="K206" s="2" t="n"/>
+      <c r="L206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
@@ -3059,6 +3499,8 @@
       <c r="H207" s="2" t="n"/>
       <c r="I207" s="2" t="n"/>
       <c r="J207" s="2" t="n"/>
+      <c r="K207" s="2" t="n"/>
+      <c r="L207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
@@ -3071,6 +3513,8 @@
       <c r="H208" s="2" t="n"/>
       <c r="I208" s="2" t="n"/>
       <c r="J208" s="2" t="n"/>
+      <c r="K208" s="2" t="n"/>
+      <c r="L208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n"/>
@@ -3083,6 +3527,8 @@
       <c r="H209" s="2" t="n"/>
       <c r="I209" s="2" t="n"/>
       <c r="J209" s="2" t="n"/>
+      <c r="K209" s="2" t="n"/>
+      <c r="L209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
@@ -3095,6 +3541,8 @@
       <c r="H210" s="2" t="n"/>
       <c r="I210" s="2" t="n"/>
       <c r="J210" s="2" t="n"/>
+      <c r="K210" s="2" t="n"/>
+      <c r="L210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n"/>
@@ -3107,6 +3555,8 @@
       <c r="H211" s="2" t="n"/>
       <c r="I211" s="2" t="n"/>
       <c r="J211" s="2" t="n"/>
+      <c r="K211" s="2" t="n"/>
+      <c r="L211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
@@ -3119,6 +3569,8 @@
       <c r="H212" s="2" t="n"/>
       <c r="I212" s="2" t="n"/>
       <c r="J212" s="2" t="n"/>
+      <c r="K212" s="2" t="n"/>
+      <c r="L212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
@@ -3131,6 +3583,8 @@
       <c r="H213" s="2" t="n"/>
       <c r="I213" s="2" t="n"/>
       <c r="J213" s="2" t="n"/>
+      <c r="K213" s="2" t="n"/>
+      <c r="L213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n"/>
@@ -3143,6 +3597,8 @@
       <c r="H214" s="2" t="n"/>
       <c r="I214" s="2" t="n"/>
       <c r="J214" s="2" t="n"/>
+      <c r="K214" s="2" t="n"/>
+      <c r="L214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n"/>
@@ -3155,6 +3611,8 @@
       <c r="H215" s="2" t="n"/>
       <c r="I215" s="2" t="n"/>
       <c r="J215" s="2" t="n"/>
+      <c r="K215" s="2" t="n"/>
+      <c r="L215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n"/>
@@ -3167,6 +3625,8 @@
       <c r="H216" s="2" t="n"/>
       <c r="I216" s="2" t="n"/>
       <c r="J216" s="2" t="n"/>
+      <c r="K216" s="2" t="n"/>
+      <c r="L216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n"/>
@@ -3179,6 +3639,8 @@
       <c r="H217" s="2" t="n"/>
       <c r="I217" s="2" t="n"/>
       <c r="J217" s="2" t="n"/>
+      <c r="K217" s="2" t="n"/>
+      <c r="L217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n"/>
@@ -3191,6 +3653,8 @@
       <c r="H218" s="2" t="n"/>
       <c r="I218" s="2" t="n"/>
       <c r="J218" s="2" t="n"/>
+      <c r="K218" s="2" t="n"/>
+      <c r="L218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n"/>
@@ -3203,6 +3667,8 @@
       <c r="H219" s="2" t="n"/>
       <c r="I219" s="2" t="n"/>
       <c r="J219" s="2" t="n"/>
+      <c r="K219" s="2" t="n"/>
+      <c r="L219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n"/>
@@ -3215,6 +3681,8 @@
       <c r="H220" s="2" t="n"/>
       <c r="I220" s="2" t="n"/>
       <c r="J220" s="2" t="n"/>
+      <c r="K220" s="2" t="n"/>
+      <c r="L220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n"/>
@@ -3227,6 +3695,8 @@
       <c r="H221" s="2" t="n"/>
       <c r="I221" s="2" t="n"/>
       <c r="J221" s="2" t="n"/>
+      <c r="K221" s="2" t="n"/>
+      <c r="L221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n"/>
@@ -3239,6 +3709,8 @@
       <c r="H222" s="2" t="n"/>
       <c r="I222" s="2" t="n"/>
       <c r="J222" s="2" t="n"/>
+      <c r="K222" s="2" t="n"/>
+      <c r="L222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n"/>
@@ -3251,6 +3723,8 @@
       <c r="H223" s="2" t="n"/>
       <c r="I223" s="2" t="n"/>
       <c r="J223" s="2" t="n"/>
+      <c r="K223" s="2" t="n"/>
+      <c r="L223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n"/>
@@ -3263,6 +3737,8 @@
       <c r="H224" s="2" t="n"/>
       <c r="I224" s="2" t="n"/>
       <c r="J224" s="2" t="n"/>
+      <c r="K224" s="2" t="n"/>
+      <c r="L224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n"/>
@@ -3275,6 +3751,8 @@
       <c r="H225" s="2" t="n"/>
       <c r="I225" s="2" t="n"/>
       <c r="J225" s="2" t="n"/>
+      <c r="K225" s="2" t="n"/>
+      <c r="L225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n"/>
@@ -3287,6 +3765,8 @@
       <c r="H226" s="2" t="n"/>
       <c r="I226" s="2" t="n"/>
       <c r="J226" s="2" t="n"/>
+      <c r="K226" s="2" t="n"/>
+      <c r="L226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n"/>
@@ -3299,6 +3779,8 @@
       <c r="H227" s="2" t="n"/>
       <c r="I227" s="2" t="n"/>
       <c r="J227" s="2" t="n"/>
+      <c r="K227" s="2" t="n"/>
+      <c r="L227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n"/>
@@ -3311,6 +3793,8 @@
       <c r="H228" s="2" t="n"/>
       <c r="I228" s="2" t="n"/>
       <c r="J228" s="2" t="n"/>
+      <c r="K228" s="2" t="n"/>
+      <c r="L228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n"/>
@@ -3323,6 +3807,8 @@
       <c r="H229" s="2" t="n"/>
       <c r="I229" s="2" t="n"/>
       <c r="J229" s="2" t="n"/>
+      <c r="K229" s="2" t="n"/>
+      <c r="L229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n"/>
@@ -3335,6 +3821,8 @@
       <c r="H230" s="2" t="n"/>
       <c r="I230" s="2" t="n"/>
       <c r="J230" s="2" t="n"/>
+      <c r="K230" s="2" t="n"/>
+      <c r="L230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n"/>
@@ -3347,6 +3835,8 @@
       <c r="H231" s="2" t="n"/>
       <c r="I231" s="2" t="n"/>
       <c r="J231" s="2" t="n"/>
+      <c r="K231" s="2" t="n"/>
+      <c r="L231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n"/>
@@ -3359,6 +3849,8 @@
       <c r="H232" s="2" t="n"/>
       <c r="I232" s="2" t="n"/>
       <c r="J232" s="2" t="n"/>
+      <c r="K232" s="2" t="n"/>
+      <c r="L232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n"/>
@@ -3371,6 +3863,8 @@
       <c r="H233" s="2" t="n"/>
       <c r="I233" s="2" t="n"/>
       <c r="J233" s="2" t="n"/>
+      <c r="K233" s="2" t="n"/>
+      <c r="L233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n"/>
@@ -3383,6 +3877,8 @@
       <c r="H234" s="2" t="n"/>
       <c r="I234" s="2" t="n"/>
       <c r="J234" s="2" t="n"/>
+      <c r="K234" s="2" t="n"/>
+      <c r="L234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n"/>
@@ -3395,6 +3891,8 @@
       <c r="H235" s="2" t="n"/>
       <c r="I235" s="2" t="n"/>
       <c r="J235" s="2" t="n"/>
+      <c r="K235" s="2" t="n"/>
+      <c r="L235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n"/>
@@ -3407,6 +3905,8 @@
       <c r="H236" s="2" t="n"/>
       <c r="I236" s="2" t="n"/>
       <c r="J236" s="2" t="n"/>
+      <c r="K236" s="2" t="n"/>
+      <c r="L236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n"/>
@@ -3419,6 +3919,8 @@
       <c r="H237" s="2" t="n"/>
       <c r="I237" s="2" t="n"/>
       <c r="J237" s="2" t="n"/>
+      <c r="K237" s="2" t="n"/>
+      <c r="L237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n"/>
@@ -3431,6 +3933,8 @@
       <c r="H238" s="2" t="n"/>
       <c r="I238" s="2" t="n"/>
       <c r="J238" s="2" t="n"/>
+      <c r="K238" s="2" t="n"/>
+      <c r="L238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n"/>
@@ -3443,6 +3947,8 @@
       <c r="H239" s="2" t="n"/>
       <c r="I239" s="2" t="n"/>
       <c r="J239" s="2" t="n"/>
+      <c r="K239" s="2" t="n"/>
+      <c r="L239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n"/>
@@ -3455,6 +3961,8 @@
       <c r="H240" s="2" t="n"/>
       <c r="I240" s="2" t="n"/>
       <c r="J240" s="2" t="n"/>
+      <c r="K240" s="2" t="n"/>
+      <c r="L240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n"/>
@@ -3467,6 +3975,8 @@
       <c r="H241" s="2" t="n"/>
       <c r="I241" s="2" t="n"/>
       <c r="J241" s="2" t="n"/>
+      <c r="K241" s="2" t="n"/>
+      <c r="L241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n"/>
@@ -3479,6 +3989,8 @@
       <c r="H242" s="2" t="n"/>
       <c r="I242" s="2" t="n"/>
       <c r="J242" s="2" t="n"/>
+      <c r="K242" s="2" t="n"/>
+      <c r="L242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n"/>
@@ -3491,6 +4003,8 @@
       <c r="H243" s="2" t="n"/>
       <c r="I243" s="2" t="n"/>
       <c r="J243" s="2" t="n"/>
+      <c r="K243" s="2" t="n"/>
+      <c r="L243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n"/>
@@ -3503,6 +4017,8 @@
       <c r="H244" s="2" t="n"/>
       <c r="I244" s="2" t="n"/>
       <c r="J244" s="2" t="n"/>
+      <c r="K244" s="2" t="n"/>
+      <c r="L244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n"/>
@@ -3515,6 +4031,8 @@
       <c r="H245" s="2" t="n"/>
       <c r="I245" s="2" t="n"/>
       <c r="J245" s="2" t="n"/>
+      <c r="K245" s="2" t="n"/>
+      <c r="L245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n"/>
@@ -3527,6 +4045,8 @@
       <c r="H246" s="2" t="n"/>
       <c r="I246" s="2" t="n"/>
       <c r="J246" s="2" t="n"/>
+      <c r="K246" s="2" t="n"/>
+      <c r="L246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n"/>
@@ -3539,6 +4059,8 @@
       <c r="H247" s="2" t="n"/>
       <c r="I247" s="2" t="n"/>
       <c r="J247" s="2" t="n"/>
+      <c r="K247" s="2" t="n"/>
+      <c r="L247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n"/>
@@ -3551,6 +4073,8 @@
       <c r="H248" s="2" t="n"/>
       <c r="I248" s="2" t="n"/>
       <c r="J248" s="2" t="n"/>
+      <c r="K248" s="2" t="n"/>
+      <c r="L248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n"/>
@@ -3563,6 +4087,8 @@
       <c r="H249" s="2" t="n"/>
       <c r="I249" s="2" t="n"/>
       <c r="J249" s="2" t="n"/>
+      <c r="K249" s="2" t="n"/>
+      <c r="L249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n"/>
@@ -3575,6 +4101,8 @@
       <c r="H250" s="2" t="n"/>
       <c r="I250" s="2" t="n"/>
       <c r="J250" s="2" t="n"/>
+      <c r="K250" s="2" t="n"/>
+      <c r="L250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n"/>
@@ -3587,6 +4115,8 @@
       <c r="H251" s="2" t="n"/>
       <c r="I251" s="2" t="n"/>
       <c r="J251" s="2" t="n"/>
+      <c r="K251" s="2" t="n"/>
+      <c r="L251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n"/>
@@ -3599,6 +4129,8 @@
       <c r="H252" s="2" t="n"/>
       <c r="I252" s="2" t="n"/>
       <c r="J252" s="2" t="n"/>
+      <c r="K252" s="2" t="n"/>
+      <c r="L252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n"/>
@@ -3611,6 +4143,8 @@
       <c r="H253" s="2" t="n"/>
       <c r="I253" s="2" t="n"/>
       <c r="J253" s="2" t="n"/>
+      <c r="K253" s="2" t="n"/>
+      <c r="L253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n"/>
@@ -3623,6 +4157,8 @@
       <c r="H254" s="2" t="n"/>
       <c r="I254" s="2" t="n"/>
       <c r="J254" s="2" t="n"/>
+      <c r="K254" s="2" t="n"/>
+      <c r="L254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n"/>
@@ -3635,6 +4171,8 @@
       <c r="H255" s="2" t="n"/>
       <c r="I255" s="2" t="n"/>
       <c r="J255" s="2" t="n"/>
+      <c r="K255" s="2" t="n"/>
+      <c r="L255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n"/>
@@ -3647,6 +4185,8 @@
       <c r="H256" s="2" t="n"/>
       <c r="I256" s="2" t="n"/>
       <c r="J256" s="2" t="n"/>
+      <c r="K256" s="2" t="n"/>
+      <c r="L256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n"/>
@@ -3659,6 +4199,8 @@
       <c r="H257" s="2" t="n"/>
       <c r="I257" s="2" t="n"/>
       <c r="J257" s="2" t="n"/>
+      <c r="K257" s="2" t="n"/>
+      <c r="L257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n"/>
@@ -3671,6 +4213,8 @@
       <c r="H258" s="2" t="n"/>
       <c r="I258" s="2" t="n"/>
       <c r="J258" s="2" t="n"/>
+      <c r="K258" s="2" t="n"/>
+      <c r="L258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n"/>
@@ -3683,6 +4227,8 @@
       <c r="H259" s="2" t="n"/>
       <c r="I259" s="2" t="n"/>
       <c r="J259" s="2" t="n"/>
+      <c r="K259" s="2" t="n"/>
+      <c r="L259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n"/>
@@ -3695,6 +4241,8 @@
       <c r="H260" s="2" t="n"/>
       <c r="I260" s="2" t="n"/>
       <c r="J260" s="2" t="n"/>
+      <c r="K260" s="2" t="n"/>
+      <c r="L260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n"/>
@@ -3707,6 +4255,8 @@
       <c r="H261" s="2" t="n"/>
       <c r="I261" s="2" t="n"/>
       <c r="J261" s="2" t="n"/>
+      <c r="K261" s="2" t="n"/>
+      <c r="L261" s="2" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n"/>
@@ -3719,6 +4269,8 @@
       <c r="H262" s="2" t="n"/>
       <c r="I262" s="2" t="n"/>
       <c r="J262" s="2" t="n"/>
+      <c r="K262" s="2" t="n"/>
+      <c r="L262" s="2" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n"/>
@@ -3731,6 +4283,8 @@
       <c r="H263" s="2" t="n"/>
       <c r="I263" s="2" t="n"/>
       <c r="J263" s="2" t="n"/>
+      <c r="K263" s="2" t="n"/>
+      <c r="L263" s="2" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n"/>
@@ -3743,6 +4297,8 @@
       <c r="H264" s="2" t="n"/>
       <c r="I264" s="2" t="n"/>
       <c r="J264" s="2" t="n"/>
+      <c r="K264" s="2" t="n"/>
+      <c r="L264" s="2" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n"/>
@@ -3755,6 +4311,8 @@
       <c r="H265" s="2" t="n"/>
       <c r="I265" s="2" t="n"/>
       <c r="J265" s="2" t="n"/>
+      <c r="K265" s="2" t="n"/>
+      <c r="L265" s="2" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n"/>
@@ -3767,6 +4325,8 @@
       <c r="H266" s="2" t="n"/>
       <c r="I266" s="2" t="n"/>
       <c r="J266" s="2" t="n"/>
+      <c r="K266" s="2" t="n"/>
+      <c r="L266" s="2" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n"/>
@@ -3779,6 +4339,8 @@
       <c r="H267" s="2" t="n"/>
       <c r="I267" s="2" t="n"/>
       <c r="J267" s="2" t="n"/>
+      <c r="K267" s="2" t="n"/>
+      <c r="L267" s="2" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n"/>
@@ -3791,6 +4353,8 @@
       <c r="H268" s="2" t="n"/>
       <c r="I268" s="2" t="n"/>
       <c r="J268" s="2" t="n"/>
+      <c r="K268" s="2" t="n"/>
+      <c r="L268" s="2" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n"/>
@@ -3803,6 +4367,8 @@
       <c r="H269" s="2" t="n"/>
       <c r="I269" s="2" t="n"/>
       <c r="J269" s="2" t="n"/>
+      <c r="K269" s="2" t="n"/>
+      <c r="L269" s="2" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n"/>
@@ -3815,6 +4381,8 @@
       <c r="H270" s="2" t="n"/>
       <c r="I270" s="2" t="n"/>
       <c r="J270" s="2" t="n"/>
+      <c r="K270" s="2" t="n"/>
+      <c r="L270" s="2" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n"/>
@@ -3827,6 +4395,8 @@
       <c r="H271" s="2" t="n"/>
       <c r="I271" s="2" t="n"/>
       <c r="J271" s="2" t="n"/>
+      <c r="K271" s="2" t="n"/>
+      <c r="L271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n"/>
@@ -3839,6 +4409,8 @@
       <c r="H272" s="2" t="n"/>
       <c r="I272" s="2" t="n"/>
       <c r="J272" s="2" t="n"/>
+      <c r="K272" s="2" t="n"/>
+      <c r="L272" s="2" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n"/>
@@ -3851,6 +4423,8 @@
       <c r="H273" s="2" t="n"/>
       <c r="I273" s="2" t="n"/>
       <c r="J273" s="2" t="n"/>
+      <c r="K273" s="2" t="n"/>
+      <c r="L273" s="2" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n"/>
@@ -3863,6 +4437,8 @@
       <c r="H274" s="2" t="n"/>
       <c r="I274" s="2" t="n"/>
       <c r="J274" s="2" t="n"/>
+      <c r="K274" s="2" t="n"/>
+      <c r="L274" s="2" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n"/>
@@ -3875,6 +4451,8 @@
       <c r="H275" s="2" t="n"/>
       <c r="I275" s="2" t="n"/>
       <c r="J275" s="2" t="n"/>
+      <c r="K275" s="2" t="n"/>
+      <c r="L275" s="2" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n"/>
@@ -3887,6 +4465,8 @@
       <c r="H276" s="2" t="n"/>
       <c r="I276" s="2" t="n"/>
       <c r="J276" s="2" t="n"/>
+      <c r="K276" s="2" t="n"/>
+      <c r="L276" s="2" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n"/>
@@ -3899,6 +4479,8 @@
       <c r="H277" s="2" t="n"/>
       <c r="I277" s="2" t="n"/>
       <c r="J277" s="2" t="n"/>
+      <c r="K277" s="2" t="n"/>
+      <c r="L277" s="2" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n"/>
@@ -3911,6 +4493,8 @@
       <c r="H278" s="2" t="n"/>
       <c r="I278" s="2" t="n"/>
       <c r="J278" s="2" t="n"/>
+      <c r="K278" s="2" t="n"/>
+      <c r="L278" s="2" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n"/>
@@ -3923,6 +4507,8 @@
       <c r="H279" s="2" t="n"/>
       <c r="I279" s="2" t="n"/>
       <c r="J279" s="2" t="n"/>
+      <c r="K279" s="2" t="n"/>
+      <c r="L279" s="2" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n"/>
@@ -3935,6 +4521,8 @@
       <c r="H280" s="2" t="n"/>
       <c r="I280" s="2" t="n"/>
       <c r="J280" s="2" t="n"/>
+      <c r="K280" s="2" t="n"/>
+      <c r="L280" s="2" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n"/>
@@ -3947,6 +4535,8 @@
       <c r="H281" s="2" t="n"/>
       <c r="I281" s="2" t="n"/>
       <c r="J281" s="2" t="n"/>
+      <c r="K281" s="2" t="n"/>
+      <c r="L281" s="2" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n"/>
@@ -3959,6 +4549,8 @@
       <c r="H282" s="2" t="n"/>
       <c r="I282" s="2" t="n"/>
       <c r="J282" s="2" t="n"/>
+      <c r="K282" s="2" t="n"/>
+      <c r="L282" s="2" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n"/>
@@ -3971,6 +4563,8 @@
       <c r="H283" s="2" t="n"/>
       <c r="I283" s="2" t="n"/>
       <c r="J283" s="2" t="n"/>
+      <c r="K283" s="2" t="n"/>
+      <c r="L283" s="2" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n"/>
@@ -3983,6 +4577,8 @@
       <c r="H284" s="2" t="n"/>
       <c r="I284" s="2" t="n"/>
       <c r="J284" s="2" t="n"/>
+      <c r="K284" s="2" t="n"/>
+      <c r="L284" s="2" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n"/>
@@ -3995,6 +4591,8 @@
       <c r="H285" s="2" t="n"/>
       <c r="I285" s="2" t="n"/>
       <c r="J285" s="2" t="n"/>
+      <c r="K285" s="2" t="n"/>
+      <c r="L285" s="2" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n"/>
@@ -4007,6 +4605,8 @@
       <c r="H286" s="2" t="n"/>
       <c r="I286" s="2" t="n"/>
       <c r="J286" s="2" t="n"/>
+      <c r="K286" s="2" t="n"/>
+      <c r="L286" s="2" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n"/>
@@ -4019,6 +4619,8 @@
       <c r="H287" s="2" t="n"/>
       <c r="I287" s="2" t="n"/>
       <c r="J287" s="2" t="n"/>
+      <c r="K287" s="2" t="n"/>
+      <c r="L287" s="2" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n"/>
@@ -4031,6 +4633,8 @@
       <c r="H288" s="2" t="n"/>
       <c r="I288" s="2" t="n"/>
       <c r="J288" s="2" t="n"/>
+      <c r="K288" s="2" t="n"/>
+      <c r="L288" s="2" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n"/>
@@ -4043,6 +4647,8 @@
       <c r="H289" s="2" t="n"/>
       <c r="I289" s="2" t="n"/>
       <c r="J289" s="2" t="n"/>
+      <c r="K289" s="2" t="n"/>
+      <c r="L289" s="2" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n"/>
@@ -4055,6 +4661,8 @@
       <c r="H290" s="2" t="n"/>
       <c r="I290" s="2" t="n"/>
       <c r="J290" s="2" t="n"/>
+      <c r="K290" s="2" t="n"/>
+      <c r="L290" s="2" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n"/>
@@ -4067,6 +4675,8 @@
       <c r="H291" s="2" t="n"/>
       <c r="I291" s="2" t="n"/>
       <c r="J291" s="2" t="n"/>
+      <c r="K291" s="2" t="n"/>
+      <c r="L291" s="2" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n"/>
@@ -4079,6 +4689,8 @@
       <c r="H292" s="2" t="n"/>
       <c r="I292" s="2" t="n"/>
       <c r="J292" s="2" t="n"/>
+      <c r="K292" s="2" t="n"/>
+      <c r="L292" s="2" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n"/>
@@ -4091,6 +4703,8 @@
       <c r="H293" s="2" t="n"/>
       <c r="I293" s="2" t="n"/>
       <c r="J293" s="2" t="n"/>
+      <c r="K293" s="2" t="n"/>
+      <c r="L293" s="2" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n"/>
@@ -4103,6 +4717,8 @@
       <c r="H294" s="2" t="n"/>
       <c r="I294" s="2" t="n"/>
       <c r="J294" s="2" t="n"/>
+      <c r="K294" s="2" t="n"/>
+      <c r="L294" s="2" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n"/>
@@ -4115,6 +4731,8 @@
       <c r="H295" s="2" t="n"/>
       <c r="I295" s="2" t="n"/>
       <c r="J295" s="2" t="n"/>
+      <c r="K295" s="2" t="n"/>
+      <c r="L295" s="2" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n"/>
@@ -4127,6 +4745,8 @@
       <c r="H296" s="2" t="n"/>
       <c r="I296" s="2" t="n"/>
       <c r="J296" s="2" t="n"/>
+      <c r="K296" s="2" t="n"/>
+      <c r="L296" s="2" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n"/>
@@ -4139,6 +4759,8 @@
       <c r="H297" s="2" t="n"/>
       <c r="I297" s="2" t="n"/>
       <c r="J297" s="2" t="n"/>
+      <c r="K297" s="2" t="n"/>
+      <c r="L297" s="2" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n"/>
@@ -4151,6 +4773,8 @@
       <c r="H298" s="2" t="n"/>
       <c r="I298" s="2" t="n"/>
       <c r="J298" s="2" t="n"/>
+      <c r="K298" s="2" t="n"/>
+      <c r="L298" s="2" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n"/>
@@ -4163,6 +4787,8 @@
       <c r="H299" s="2" t="n"/>
       <c r="I299" s="2" t="n"/>
       <c r="J299" s="2" t="n"/>
+      <c r="K299" s="2" t="n"/>
+      <c r="L299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n"/>
@@ -4175,6 +4801,8 @@
       <c r="H300" s="2" t="n"/>
       <c r="I300" s="2" t="n"/>
       <c r="J300" s="2" t="n"/>
+      <c r="K300" s="2" t="n"/>
+      <c r="L300" s="2" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n"/>
@@ -4187,6 +4815,8 @@
       <c r="H301" s="2" t="n"/>
       <c r="I301" s="2" t="n"/>
       <c r="J301" s="2" t="n"/>
+      <c r="K301" s="2" t="n"/>
+      <c r="L301" s="2" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="n"/>
@@ -4199,6 +4829,8 @@
       <c r="H302" s="2" t="n"/>
       <c r="I302" s="2" t="n"/>
       <c r="J302" s="2" t="n"/>
+      <c r="K302" s="2" t="n"/>
+      <c r="L302" s="2" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="n"/>
@@ -4211,6 +4843,8 @@
       <c r="H303" s="2" t="n"/>
       <c r="I303" s="2" t="n"/>
       <c r="J303" s="2" t="n"/>
+      <c r="K303" s="2" t="n"/>
+      <c r="L303" s="2" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="n"/>
@@ -4223,6 +4857,8 @@
       <c r="H304" s="2" t="n"/>
       <c r="I304" s="2" t="n"/>
       <c r="J304" s="2" t="n"/>
+      <c r="K304" s="2" t="n"/>
+      <c r="L304" s="2" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="n"/>
@@ -4235,6 +4871,8 @@
       <c r="H305" s="2" t="n"/>
       <c r="I305" s="2" t="n"/>
       <c r="J305" s="2" t="n"/>
+      <c r="K305" s="2" t="n"/>
+      <c r="L305" s="2" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="n"/>
@@ -4247,6 +4885,8 @@
       <c r="H306" s="2" t="n"/>
       <c r="I306" s="2" t="n"/>
       <c r="J306" s="2" t="n"/>
+      <c r="K306" s="2" t="n"/>
+      <c r="L306" s="2" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="n"/>
@@ -4259,6 +4899,8 @@
       <c r="H307" s="2" t="n"/>
       <c r="I307" s="2" t="n"/>
       <c r="J307" s="2" t="n"/>
+      <c r="K307" s="2" t="n"/>
+      <c r="L307" s="2" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="n"/>
@@ -4271,6 +4913,8 @@
       <c r="H308" s="2" t="n"/>
       <c r="I308" s="2" t="n"/>
       <c r="J308" s="2" t="n"/>
+      <c r="K308" s="2" t="n"/>
+      <c r="L308" s="2" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="n"/>
@@ -4283,6 +4927,8 @@
       <c r="H309" s="2" t="n"/>
       <c r="I309" s="2" t="n"/>
       <c r="J309" s="2" t="n"/>
+      <c r="K309" s="2" t="n"/>
+      <c r="L309" s="2" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="n"/>
@@ -4295,6 +4941,8 @@
       <c r="H310" s="2" t="n"/>
       <c r="I310" s="2" t="n"/>
       <c r="J310" s="2" t="n"/>
+      <c r="K310" s="2" t="n"/>
+      <c r="L310" s="2" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="n"/>
@@ -4307,6 +4955,8 @@
       <c r="H311" s="2" t="n"/>
       <c r="I311" s="2" t="n"/>
       <c r="J311" s="2" t="n"/>
+      <c r="K311" s="2" t="n"/>
+      <c r="L311" s="2" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="n"/>
@@ -4319,6 +4969,8 @@
       <c r="H312" s="2" t="n"/>
       <c r="I312" s="2" t="n"/>
       <c r="J312" s="2" t="n"/>
+      <c r="K312" s="2" t="n"/>
+      <c r="L312" s="2" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="n"/>
@@ -4331,6 +4983,8 @@
       <c r="H313" s="2" t="n"/>
       <c r="I313" s="2" t="n"/>
       <c r="J313" s="2" t="n"/>
+      <c r="K313" s="2" t="n"/>
+      <c r="L313" s="2" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="n"/>
@@ -4343,6 +4997,8 @@
       <c r="H314" s="2" t="n"/>
       <c r="I314" s="2" t="n"/>
       <c r="J314" s="2" t="n"/>
+      <c r="K314" s="2" t="n"/>
+      <c r="L314" s="2" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="n"/>
@@ -4355,6 +5011,8 @@
       <c r="H315" s="2" t="n"/>
       <c r="I315" s="2" t="n"/>
       <c r="J315" s="2" t="n"/>
+      <c r="K315" s="2" t="n"/>
+      <c r="L315" s="2" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="n"/>
@@ -4367,6 +5025,8 @@
       <c r="H316" s="2" t="n"/>
       <c r="I316" s="2" t="n"/>
       <c r="J316" s="2" t="n"/>
+      <c r="K316" s="2" t="n"/>
+      <c r="L316" s="2" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="n"/>
@@ -4379,6 +5039,8 @@
       <c r="H317" s="2" t="n"/>
       <c r="I317" s="2" t="n"/>
       <c r="J317" s="2" t="n"/>
+      <c r="K317" s="2" t="n"/>
+      <c r="L317" s="2" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="n"/>
@@ -4391,6 +5053,8 @@
       <c r="H318" s="2" t="n"/>
       <c r="I318" s="2" t="n"/>
       <c r="J318" s="2" t="n"/>
+      <c r="K318" s="2" t="n"/>
+      <c r="L318" s="2" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="n"/>
@@ -4403,6 +5067,8 @@
       <c r="H319" s="2" t="n"/>
       <c r="I319" s="2" t="n"/>
       <c r="J319" s="2" t="n"/>
+      <c r="K319" s="2" t="n"/>
+      <c r="L319" s="2" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="n"/>
@@ -4415,6 +5081,8 @@
       <c r="H320" s="2" t="n"/>
       <c r="I320" s="2" t="n"/>
       <c r="J320" s="2" t="n"/>
+      <c r="K320" s="2" t="n"/>
+      <c r="L320" s="2" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="n"/>
@@ -4427,6 +5095,8 @@
       <c r="H321" s="2" t="n"/>
       <c r="I321" s="2" t="n"/>
       <c r="J321" s="2" t="n"/>
+      <c r="K321" s="2" t="n"/>
+      <c r="L321" s="2" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="n"/>
@@ -4439,6 +5109,8 @@
       <c r="H322" s="2" t="n"/>
       <c r="I322" s="2" t="n"/>
       <c r="J322" s="2" t="n"/>
+      <c r="K322" s="2" t="n"/>
+      <c r="L322" s="2" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="n"/>
@@ -4451,6 +5123,8 @@
       <c r="H323" s="2" t="n"/>
       <c r="I323" s="2" t="n"/>
       <c r="J323" s="2" t="n"/>
+      <c r="K323" s="2" t="n"/>
+      <c r="L323" s="2" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="2" t="n"/>
@@ -4463,6 +5137,8 @@
       <c r="H324" s="2" t="n"/>
       <c r="I324" s="2" t="n"/>
       <c r="J324" s="2" t="n"/>
+      <c r="K324" s="2" t="n"/>
+      <c r="L324" s="2" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="n"/>
@@ -4475,6 +5151,8 @@
       <c r="H325" s="2" t="n"/>
       <c r="I325" s="2" t="n"/>
       <c r="J325" s="2" t="n"/>
+      <c r="K325" s="2" t="n"/>
+      <c r="L325" s="2" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="n"/>
@@ -4487,6 +5165,8 @@
       <c r="H326" s="2" t="n"/>
       <c r="I326" s="2" t="n"/>
       <c r="J326" s="2" t="n"/>
+      <c r="K326" s="2" t="n"/>
+      <c r="L326" s="2" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="n"/>
@@ -4499,6 +5179,8 @@
       <c r="H327" s="2" t="n"/>
       <c r="I327" s="2" t="n"/>
       <c r="J327" s="2" t="n"/>
+      <c r="K327" s="2" t="n"/>
+      <c r="L327" s="2" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="n"/>
@@ -4511,6 +5193,8 @@
       <c r="H328" s="2" t="n"/>
       <c r="I328" s="2" t="n"/>
       <c r="J328" s="2" t="n"/>
+      <c r="K328" s="2" t="n"/>
+      <c r="L328" s="2" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="n"/>
@@ -4523,6 +5207,8 @@
       <c r="H329" s="2" t="n"/>
       <c r="I329" s="2" t="n"/>
       <c r="J329" s="2" t="n"/>
+      <c r="K329" s="2" t="n"/>
+      <c r="L329" s="2" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="n"/>
@@ -4535,6 +5221,8 @@
       <c r="H330" s="2" t="n"/>
       <c r="I330" s="2" t="n"/>
       <c r="J330" s="2" t="n"/>
+      <c r="K330" s="2" t="n"/>
+      <c r="L330" s="2" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="n"/>
@@ -4547,6 +5235,8 @@
       <c r="H331" s="2" t="n"/>
       <c r="I331" s="2" t="n"/>
       <c r="J331" s="2" t="n"/>
+      <c r="K331" s="2" t="n"/>
+      <c r="L331" s="2" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="n"/>
@@ -4559,6 +5249,8 @@
       <c r="H332" s="2" t="n"/>
       <c r="I332" s="2" t="n"/>
       <c r="J332" s="2" t="n"/>
+      <c r="K332" s="2" t="n"/>
+      <c r="L332" s="2" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="n"/>
@@ -4571,6 +5263,8 @@
       <c r="H333" s="2" t="n"/>
       <c r="I333" s="2" t="n"/>
       <c r="J333" s="2" t="n"/>
+      <c r="K333" s="2" t="n"/>
+      <c r="L333" s="2" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="n"/>
@@ -4583,6 +5277,8 @@
       <c r="H334" s="2" t="n"/>
       <c r="I334" s="2" t="n"/>
       <c r="J334" s="2" t="n"/>
+      <c r="K334" s="2" t="n"/>
+      <c r="L334" s="2" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="n"/>
@@ -4595,6 +5291,8 @@
       <c r="H335" s="2" t="n"/>
       <c r="I335" s="2" t="n"/>
       <c r="J335" s="2" t="n"/>
+      <c r="K335" s="2" t="n"/>
+      <c r="L335" s="2" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="n"/>
@@ -4607,6 +5305,8 @@
       <c r="H336" s="2" t="n"/>
       <c r="I336" s="2" t="n"/>
       <c r="J336" s="2" t="n"/>
+      <c r="K336" s="2" t="n"/>
+      <c r="L336" s="2" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="n"/>
@@ -4619,6 +5319,8 @@
       <c r="H337" s="2" t="n"/>
       <c r="I337" s="2" t="n"/>
       <c r="J337" s="2" t="n"/>
+      <c r="K337" s="2" t="n"/>
+      <c r="L337" s="2" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="n"/>
@@ -4631,6 +5333,8 @@
       <c r="H338" s="2" t="n"/>
       <c r="I338" s="2" t="n"/>
       <c r="J338" s="2" t="n"/>
+      <c r="K338" s="2" t="n"/>
+      <c r="L338" s="2" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="n"/>
@@ -4643,6 +5347,8 @@
       <c r="H339" s="2" t="n"/>
       <c r="I339" s="2" t="n"/>
       <c r="J339" s="2" t="n"/>
+      <c r="K339" s="2" t="n"/>
+      <c r="L339" s="2" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="n"/>
@@ -4655,6 +5361,8 @@
       <c r="H340" s="2" t="n"/>
       <c r="I340" s="2" t="n"/>
       <c r="J340" s="2" t="n"/>
+      <c r="K340" s="2" t="n"/>
+      <c r="L340" s="2" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="n"/>
@@ -4667,6 +5375,8 @@
       <c r="H341" s="2" t="n"/>
       <c r="I341" s="2" t="n"/>
       <c r="J341" s="2" t="n"/>
+      <c r="K341" s="2" t="n"/>
+      <c r="L341" s="2" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="n"/>
@@ -4679,6 +5389,8 @@
       <c r="H342" s="2" t="n"/>
       <c r="I342" s="2" t="n"/>
       <c r="J342" s="2" t="n"/>
+      <c r="K342" s="2" t="n"/>
+      <c r="L342" s="2" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="n"/>
@@ -4691,6 +5403,8 @@
       <c r="H343" s="2" t="n"/>
       <c r="I343" s="2" t="n"/>
       <c r="J343" s="2" t="n"/>
+      <c r="K343" s="2" t="n"/>
+      <c r="L343" s="2" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="2" t="n"/>
@@ -4703,6 +5417,8 @@
       <c r="H344" s="2" t="n"/>
       <c r="I344" s="2" t="n"/>
       <c r="J344" s="2" t="n"/>
+      <c r="K344" s="2" t="n"/>
+      <c r="L344" s="2" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="n"/>
@@ -4715,6 +5431,8 @@
       <c r="H345" s="2" t="n"/>
       <c r="I345" s="2" t="n"/>
       <c r="J345" s="2" t="n"/>
+      <c r="K345" s="2" t="n"/>
+      <c r="L345" s="2" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="n"/>
@@ -4727,6 +5445,8 @@
       <c r="H346" s="2" t="n"/>
       <c r="I346" s="2" t="n"/>
       <c r="J346" s="2" t="n"/>
+      <c r="K346" s="2" t="n"/>
+      <c r="L346" s="2" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n"/>
@@ -4739,6 +5459,8 @@
       <c r="H347" s="2" t="n"/>
       <c r="I347" s="2" t="n"/>
       <c r="J347" s="2" t="n"/>
+      <c r="K347" s="2" t="n"/>
+      <c r="L347" s="2" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n"/>
@@ -4751,6 +5473,8 @@
       <c r="H348" s="2" t="n"/>
       <c r="I348" s="2" t="n"/>
       <c r="J348" s="2" t="n"/>
+      <c r="K348" s="2" t="n"/>
+      <c r="L348" s="2" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n"/>
@@ -4763,6 +5487,8 @@
       <c r="H349" s="2" t="n"/>
       <c r="I349" s="2" t="n"/>
       <c r="J349" s="2" t="n"/>
+      <c r="K349" s="2" t="n"/>
+      <c r="L349" s="2" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n"/>
@@ -4775,6 +5501,8 @@
       <c r="H350" s="2" t="n"/>
       <c r="I350" s="2" t="n"/>
       <c r="J350" s="2" t="n"/>
+      <c r="K350" s="2" t="n"/>
+      <c r="L350" s="2" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n"/>
@@ -4787,6 +5515,8 @@
       <c r="H351" s="2" t="n"/>
       <c r="I351" s="2" t="n"/>
       <c r="J351" s="2" t="n"/>
+      <c r="K351" s="2" t="n"/>
+      <c r="L351" s="2" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n"/>
@@ -4799,6 +5529,8 @@
       <c r="H352" s="2" t="n"/>
       <c r="I352" s="2" t="n"/>
       <c r="J352" s="2" t="n"/>
+      <c r="K352" s="2" t="n"/>
+      <c r="L352" s="2" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n"/>
@@ -4811,6 +5543,8 @@
       <c r="H353" s="2" t="n"/>
       <c r="I353" s="2" t="n"/>
       <c r="J353" s="2" t="n"/>
+      <c r="K353" s="2" t="n"/>
+      <c r="L353" s="2" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n"/>
@@ -4823,6 +5557,8 @@
       <c r="H354" s="2" t="n"/>
       <c r="I354" s="2" t="n"/>
       <c r="J354" s="2" t="n"/>
+      <c r="K354" s="2" t="n"/>
+      <c r="L354" s="2" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n"/>
@@ -4835,6 +5571,8 @@
       <c r="H355" s="2" t="n"/>
       <c r="I355" s="2" t="n"/>
       <c r="J355" s="2" t="n"/>
+      <c r="K355" s="2" t="n"/>
+      <c r="L355" s="2" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n"/>
@@ -4847,6 +5585,8 @@
       <c r="H356" s="2" t="n"/>
       <c r="I356" s="2" t="n"/>
       <c r="J356" s="2" t="n"/>
+      <c r="K356" s="2" t="n"/>
+      <c r="L356" s="2" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n"/>
@@ -4859,6 +5599,8 @@
       <c r="H357" s="2" t="n"/>
       <c r="I357" s="2" t="n"/>
       <c r="J357" s="2" t="n"/>
+      <c r="K357" s="2" t="n"/>
+      <c r="L357" s="2" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n"/>
@@ -4871,6 +5613,8 @@
       <c r="H358" s="2" t="n"/>
       <c r="I358" s="2" t="n"/>
       <c r="J358" s="2" t="n"/>
+      <c r="K358" s="2" t="n"/>
+      <c r="L358" s="2" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="n"/>
@@ -4883,6 +5627,8 @@
       <c r="H359" s="2" t="n"/>
       <c r="I359" s="2" t="n"/>
       <c r="J359" s="2" t="n"/>
+      <c r="K359" s="2" t="n"/>
+      <c r="L359" s="2" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n"/>
@@ -4895,6 +5641,8 @@
       <c r="H360" s="2" t="n"/>
       <c r="I360" s="2" t="n"/>
       <c r="J360" s="2" t="n"/>
+      <c r="K360" s="2" t="n"/>
+      <c r="L360" s="2" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n"/>
@@ -4907,6 +5655,8 @@
       <c r="H361" s="2" t="n"/>
       <c r="I361" s="2" t="n"/>
       <c r="J361" s="2" t="n"/>
+      <c r="K361" s="2" t="n"/>
+      <c r="L361" s="2" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n"/>
@@ -4919,6 +5669,8 @@
       <c r="H362" s="2" t="n"/>
       <c r="I362" s="2" t="n"/>
       <c r="J362" s="2" t="n"/>
+      <c r="K362" s="2" t="n"/>
+      <c r="L362" s="2" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n"/>
@@ -4931,6 +5683,8 @@
       <c r="H363" s="2" t="n"/>
       <c r="I363" s="2" t="n"/>
       <c r="J363" s="2" t="n"/>
+      <c r="K363" s="2" t="n"/>
+      <c r="L363" s="2" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n"/>
@@ -4943,6 +5697,8 @@
       <c r="H364" s="2" t="n"/>
       <c r="I364" s="2" t="n"/>
       <c r="J364" s="2" t="n"/>
+      <c r="K364" s="2" t="n"/>
+      <c r="L364" s="2" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="n"/>
@@ -4955,6 +5711,8 @@
       <c r="H365" s="2" t="n"/>
       <c r="I365" s="2" t="n"/>
       <c r="J365" s="2" t="n"/>
+      <c r="K365" s="2" t="n"/>
+      <c r="L365" s="2" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="n"/>
@@ -4967,6 +5725,8 @@
       <c r="H366" s="2" t="n"/>
       <c r="I366" s="2" t="n"/>
       <c r="J366" s="2" t="n"/>
+      <c r="K366" s="2" t="n"/>
+      <c r="L366" s="2" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n"/>
@@ -4979,6 +5739,8 @@
       <c r="H367" s="2" t="n"/>
       <c r="I367" s="2" t="n"/>
       <c r="J367" s="2" t="n"/>
+      <c r="K367" s="2" t="n"/>
+      <c r="L367" s="2" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n"/>
@@ -4991,6 +5753,8 @@
       <c r="H368" s="2" t="n"/>
       <c r="I368" s="2" t="n"/>
       <c r="J368" s="2" t="n"/>
+      <c r="K368" s="2" t="n"/>
+      <c r="L368" s="2" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n"/>
@@ -5003,6 +5767,8 @@
       <c r="H369" s="2" t="n"/>
       <c r="I369" s="2" t="n"/>
       <c r="J369" s="2" t="n"/>
+      <c r="K369" s="2" t="n"/>
+      <c r="L369" s="2" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n"/>
@@ -5015,6 +5781,8 @@
       <c r="H370" s="2" t="n"/>
       <c r="I370" s="2" t="n"/>
       <c r="J370" s="2" t="n"/>
+      <c r="K370" s="2" t="n"/>
+      <c r="L370" s="2" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n"/>
@@ -5027,6 +5795,8 @@
       <c r="H371" s="2" t="n"/>
       <c r="I371" s="2" t="n"/>
       <c r="J371" s="2" t="n"/>
+      <c r="K371" s="2" t="n"/>
+      <c r="L371" s="2" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n"/>
@@ -5039,6 +5809,8 @@
       <c r="H372" s="2" t="n"/>
       <c r="I372" s="2" t="n"/>
       <c r="J372" s="2" t="n"/>
+      <c r="K372" s="2" t="n"/>
+      <c r="L372" s="2" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n"/>
@@ -5051,6 +5823,8 @@
       <c r="H373" s="2" t="n"/>
       <c r="I373" s="2" t="n"/>
       <c r="J373" s="2" t="n"/>
+      <c r="K373" s="2" t="n"/>
+      <c r="L373" s="2" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n"/>
@@ -5063,6 +5837,8 @@
       <c r="H374" s="2" t="n"/>
       <c r="I374" s="2" t="n"/>
       <c r="J374" s="2" t="n"/>
+      <c r="K374" s="2" t="n"/>
+      <c r="L374" s="2" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n"/>
@@ -5075,6 +5851,8 @@
       <c r="H375" s="2" t="n"/>
       <c r="I375" s="2" t="n"/>
       <c r="J375" s="2" t="n"/>
+      <c r="K375" s="2" t="n"/>
+      <c r="L375" s="2" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n"/>
@@ -5087,6 +5865,8 @@
       <c r="H376" s="2" t="n"/>
       <c r="I376" s="2" t="n"/>
       <c r="J376" s="2" t="n"/>
+      <c r="K376" s="2" t="n"/>
+      <c r="L376" s="2" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n"/>
@@ -5099,6 +5879,8 @@
       <c r="H377" s="2" t="n"/>
       <c r="I377" s="2" t="n"/>
       <c r="J377" s="2" t="n"/>
+      <c r="K377" s="2" t="n"/>
+      <c r="L377" s="2" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n"/>
@@ -5111,6 +5893,8 @@
       <c r="H378" s="2" t="n"/>
       <c r="I378" s="2" t="n"/>
       <c r="J378" s="2" t="n"/>
+      <c r="K378" s="2" t="n"/>
+      <c r="L378" s="2" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n"/>
@@ -5123,6 +5907,8 @@
       <c r="H379" s="2" t="n"/>
       <c r="I379" s="2" t="n"/>
       <c r="J379" s="2" t="n"/>
+      <c r="K379" s="2" t="n"/>
+      <c r="L379" s="2" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n"/>
@@ -5135,6 +5921,8 @@
       <c r="H380" s="2" t="n"/>
       <c r="I380" s="2" t="n"/>
       <c r="J380" s="2" t="n"/>
+      <c r="K380" s="2" t="n"/>
+      <c r="L380" s="2" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n"/>
@@ -5147,6 +5935,8 @@
       <c r="H381" s="2" t="n"/>
       <c r="I381" s="2" t="n"/>
       <c r="J381" s="2" t="n"/>
+      <c r="K381" s="2" t="n"/>
+      <c r="L381" s="2" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n"/>
@@ -5159,6 +5949,8 @@
       <c r="H382" s="2" t="n"/>
       <c r="I382" s="2" t="n"/>
       <c r="J382" s="2" t="n"/>
+      <c r="K382" s="2" t="n"/>
+      <c r="L382" s="2" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n"/>
@@ -5171,6 +5963,8 @@
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="n"/>
       <c r="J383" s="2" t="n"/>
+      <c r="K383" s="2" t="n"/>
+      <c r="L383" s="2" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n"/>
@@ -5183,6 +5977,8 @@
       <c r="H384" s="2" t="n"/>
       <c r="I384" s="2" t="n"/>
       <c r="J384" s="2" t="n"/>
+      <c r="K384" s="2" t="n"/>
+      <c r="L384" s="2" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n"/>
@@ -5195,6 +5991,8 @@
       <c r="H385" s="2" t="n"/>
       <c r="I385" s="2" t="n"/>
       <c r="J385" s="2" t="n"/>
+      <c r="K385" s="2" t="n"/>
+      <c r="L385" s="2" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="n"/>
@@ -5207,6 +6005,8 @@
       <c r="H386" s="2" t="n"/>
       <c r="I386" s="2" t="n"/>
       <c r="J386" s="2" t="n"/>
+      <c r="K386" s="2" t="n"/>
+      <c r="L386" s="2" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="n"/>
@@ -5219,6 +6019,8 @@
       <c r="H387" s="2" t="n"/>
       <c r="I387" s="2" t="n"/>
       <c r="J387" s="2" t="n"/>
+      <c r="K387" s="2" t="n"/>
+      <c r="L387" s="2" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="n"/>
@@ -5231,6 +6033,8 @@
       <c r="H388" s="2" t="n"/>
       <c r="I388" s="2" t="n"/>
       <c r="J388" s="2" t="n"/>
+      <c r="K388" s="2" t="n"/>
+      <c r="L388" s="2" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="n"/>
@@ -5243,6 +6047,8 @@
       <c r="H389" s="2" t="n"/>
       <c r="I389" s="2" t="n"/>
       <c r="J389" s="2" t="n"/>
+      <c r="K389" s="2" t="n"/>
+      <c r="L389" s="2" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="n"/>
@@ -5255,6 +6061,8 @@
       <c r="H390" s="2" t="n"/>
       <c r="I390" s="2" t="n"/>
       <c r="J390" s="2" t="n"/>
+      <c r="K390" s="2" t="n"/>
+      <c r="L390" s="2" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="n"/>
@@ -5267,6 +6075,8 @@
       <c r="H391" s="2" t="n"/>
       <c r="I391" s="2" t="n"/>
       <c r="J391" s="2" t="n"/>
+      <c r="K391" s="2" t="n"/>
+      <c r="L391" s="2" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n"/>
@@ -5279,6 +6089,8 @@
       <c r="H392" s="2" t="n"/>
       <c r="I392" s="2" t="n"/>
       <c r="J392" s="2" t="n"/>
+      <c r="K392" s="2" t="n"/>
+      <c r="L392" s="2" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n"/>
@@ -5291,6 +6103,8 @@
       <c r="H393" s="2" t="n"/>
       <c r="I393" s="2" t="n"/>
       <c r="J393" s="2" t="n"/>
+      <c r="K393" s="2" t="n"/>
+      <c r="L393" s="2" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n"/>
@@ -5303,6 +6117,8 @@
       <c r="H394" s="2" t="n"/>
       <c r="I394" s="2" t="n"/>
       <c r="J394" s="2" t="n"/>
+      <c r="K394" s="2" t="n"/>
+      <c r="L394" s="2" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n"/>
@@ -5315,6 +6131,8 @@
       <c r="H395" s="2" t="n"/>
       <c r="I395" s="2" t="n"/>
       <c r="J395" s="2" t="n"/>
+      <c r="K395" s="2" t="n"/>
+      <c r="L395" s="2" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n"/>
@@ -5327,6 +6145,8 @@
       <c r="H396" s="2" t="n"/>
       <c r="I396" s="2" t="n"/>
       <c r="J396" s="2" t="n"/>
+      <c r="K396" s="2" t="n"/>
+      <c r="L396" s="2" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n"/>
@@ -5339,6 +6159,8 @@
       <c r="H397" s="2" t="n"/>
       <c r="I397" s="2" t="n"/>
       <c r="J397" s="2" t="n"/>
+      <c r="K397" s="2" t="n"/>
+      <c r="L397" s="2" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n"/>
@@ -5351,6 +6173,8 @@
       <c r="H398" s="2" t="n"/>
       <c r="I398" s="2" t="n"/>
       <c r="J398" s="2" t="n"/>
+      <c r="K398" s="2" t="n"/>
+      <c r="L398" s="2" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n"/>
@@ -5363,6 +6187,8 @@
       <c r="H399" s="2" t="n"/>
       <c r="I399" s="2" t="n"/>
       <c r="J399" s="2" t="n"/>
+      <c r="K399" s="2" t="n"/>
+      <c r="L399" s="2" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n"/>
@@ -5375,6 +6201,8 @@
       <c r="H400" s="2" t="n"/>
       <c r="I400" s="2" t="n"/>
       <c r="J400" s="2" t="n"/>
+      <c r="K400" s="2" t="n"/>
+      <c r="L400" s="2" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n"/>
@@ -5387,6 +6215,8 @@
       <c r="H401" s="2" t="n"/>
       <c r="I401" s="2" t="n"/>
       <c r="J401" s="2" t="n"/>
+      <c r="K401" s="2" t="n"/>
+      <c r="L401" s="2" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n"/>
@@ -5399,6 +6229,8 @@
       <c r="H402" s="2" t="n"/>
       <c r="I402" s="2" t="n"/>
       <c r="J402" s="2" t="n"/>
+      <c r="K402" s="2" t="n"/>
+      <c r="L402" s="2" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n"/>
@@ -5411,6 +6243,8 @@
       <c r="H403" s="2" t="n"/>
       <c r="I403" s="2" t="n"/>
       <c r="J403" s="2" t="n"/>
+      <c r="K403" s="2" t="n"/>
+      <c r="L403" s="2" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n"/>
@@ -5423,6 +6257,8 @@
       <c r="H404" s="2" t="n"/>
       <c r="I404" s="2" t="n"/>
       <c r="J404" s="2" t="n"/>
+      <c r="K404" s="2" t="n"/>
+      <c r="L404" s="2" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n"/>
@@ -5435,6 +6271,8 @@
       <c r="H405" s="2" t="n"/>
       <c r="I405" s="2" t="n"/>
       <c r="J405" s="2" t="n"/>
+      <c r="K405" s="2" t="n"/>
+      <c r="L405" s="2" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n"/>
@@ -5447,6 +6285,8 @@
       <c r="H406" s="2" t="n"/>
       <c r="I406" s="2" t="n"/>
       <c r="J406" s="2" t="n"/>
+      <c r="K406" s="2" t="n"/>
+      <c r="L406" s="2" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n"/>
@@ -5459,6 +6299,8 @@
       <c r="H407" s="2" t="n"/>
       <c r="I407" s="2" t="n"/>
       <c r="J407" s="2" t="n"/>
+      <c r="K407" s="2" t="n"/>
+      <c r="L407" s="2" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n"/>
@@ -5471,6 +6313,8 @@
       <c r="H408" s="2" t="n"/>
       <c r="I408" s="2" t="n"/>
       <c r="J408" s="2" t="n"/>
+      <c r="K408" s="2" t="n"/>
+      <c r="L408" s="2" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n"/>
@@ -5483,6 +6327,8 @@
       <c r="H409" s="2" t="n"/>
       <c r="I409" s="2" t="n"/>
       <c r="J409" s="2" t="n"/>
+      <c r="K409" s="2" t="n"/>
+      <c r="L409" s="2" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n"/>
@@ -5495,6 +6341,8 @@
       <c r="H410" s="2" t="n"/>
       <c r="I410" s="2" t="n"/>
       <c r="J410" s="2" t="n"/>
+      <c r="K410" s="2" t="n"/>
+      <c r="L410" s="2" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n"/>
@@ -5507,6 +6355,8 @@
       <c r="H411" s="2" t="n"/>
       <c r="I411" s="2" t="n"/>
       <c r="J411" s="2" t="n"/>
+      <c r="K411" s="2" t="n"/>
+      <c r="L411" s="2" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n"/>
@@ -5519,6 +6369,8 @@
       <c r="H412" s="2" t="n"/>
       <c r="I412" s="2" t="n"/>
       <c r="J412" s="2" t="n"/>
+      <c r="K412" s="2" t="n"/>
+      <c r="L412" s="2" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n"/>
@@ -5531,6 +6383,8 @@
       <c r="H413" s="2" t="n"/>
       <c r="I413" s="2" t="n"/>
       <c r="J413" s="2" t="n"/>
+      <c r="K413" s="2" t="n"/>
+      <c r="L413" s="2" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n"/>
@@ -5543,6 +6397,8 @@
       <c r="H414" s="2" t="n"/>
       <c r="I414" s="2" t="n"/>
       <c r="J414" s="2" t="n"/>
+      <c r="K414" s="2" t="n"/>
+      <c r="L414" s="2" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n"/>
@@ -5555,6 +6411,8 @@
       <c r="H415" s="2" t="n"/>
       <c r="I415" s="2" t="n"/>
       <c r="J415" s="2" t="n"/>
+      <c r="K415" s="2" t="n"/>
+      <c r="L415" s="2" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n"/>
@@ -5567,6 +6425,8 @@
       <c r="H416" s="2" t="n"/>
       <c r="I416" s="2" t="n"/>
       <c r="J416" s="2" t="n"/>
+      <c r="K416" s="2" t="n"/>
+      <c r="L416" s="2" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n"/>
@@ -5579,6 +6439,8 @@
       <c r="H417" s="2" t="n"/>
       <c r="I417" s="2" t="n"/>
       <c r="J417" s="2" t="n"/>
+      <c r="K417" s="2" t="n"/>
+      <c r="L417" s="2" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n"/>
@@ -5591,6 +6453,8 @@
       <c r="H418" s="2" t="n"/>
       <c r="I418" s="2" t="n"/>
       <c r="J418" s="2" t="n"/>
+      <c r="K418" s="2" t="n"/>
+      <c r="L418" s="2" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n"/>
@@ -5603,6 +6467,8 @@
       <c r="H419" s="2" t="n"/>
       <c r="I419" s="2" t="n"/>
       <c r="J419" s="2" t="n"/>
+      <c r="K419" s="2" t="n"/>
+      <c r="L419" s="2" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n"/>
@@ -5615,6 +6481,8 @@
       <c r="H420" s="2" t="n"/>
       <c r="I420" s="2" t="n"/>
       <c r="J420" s="2" t="n"/>
+      <c r="K420" s="2" t="n"/>
+      <c r="L420" s="2" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n"/>
@@ -5627,6 +6495,8 @@
       <c r="H421" s="2" t="n"/>
       <c r="I421" s="2" t="n"/>
       <c r="J421" s="2" t="n"/>
+      <c r="K421" s="2" t="n"/>
+      <c r="L421" s="2" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n"/>
@@ -5639,6 +6509,8 @@
       <c r="H422" s="2" t="n"/>
       <c r="I422" s="2" t="n"/>
       <c r="J422" s="2" t="n"/>
+      <c r="K422" s="2" t="n"/>
+      <c r="L422" s="2" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n"/>
@@ -5651,6 +6523,8 @@
       <c r="H423" s="2" t="n"/>
       <c r="I423" s="2" t="n"/>
       <c r="J423" s="2" t="n"/>
+      <c r="K423" s="2" t="n"/>
+      <c r="L423" s="2" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n"/>
@@ -5663,6 +6537,8 @@
       <c r="H424" s="2" t="n"/>
       <c r="I424" s="2" t="n"/>
       <c r="J424" s="2" t="n"/>
+      <c r="K424" s="2" t="n"/>
+      <c r="L424" s="2" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n"/>
@@ -5675,6 +6551,8 @@
       <c r="H425" s="2" t="n"/>
       <c r="I425" s="2" t="n"/>
       <c r="J425" s="2" t="n"/>
+      <c r="K425" s="2" t="n"/>
+      <c r="L425" s="2" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n"/>
@@ -5687,6 +6565,8 @@
       <c r="H426" s="2" t="n"/>
       <c r="I426" s="2" t="n"/>
       <c r="J426" s="2" t="n"/>
+      <c r="K426" s="2" t="n"/>
+      <c r="L426" s="2" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n"/>
@@ -5699,6 +6579,8 @@
       <c r="H427" s="2" t="n"/>
       <c r="I427" s="2" t="n"/>
       <c r="J427" s="2" t="n"/>
+      <c r="K427" s="2" t="n"/>
+      <c r="L427" s="2" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n"/>
@@ -5711,6 +6593,8 @@
       <c r="H428" s="2" t="n"/>
       <c r="I428" s="2" t="n"/>
       <c r="J428" s="2" t="n"/>
+      <c r="K428" s="2" t="n"/>
+      <c r="L428" s="2" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n"/>
@@ -5723,6 +6607,8 @@
       <c r="H429" s="2" t="n"/>
       <c r="I429" s="2" t="n"/>
       <c r="J429" s="2" t="n"/>
+      <c r="K429" s="2" t="n"/>
+      <c r="L429" s="2" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n"/>
@@ -5735,6 +6621,8 @@
       <c r="H430" s="2" t="n"/>
       <c r="I430" s="2" t="n"/>
       <c r="J430" s="2" t="n"/>
+      <c r="K430" s="2" t="n"/>
+      <c r="L430" s="2" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n"/>
@@ -5747,6 +6635,8 @@
       <c r="H431" s="2" t="n"/>
       <c r="I431" s="2" t="n"/>
       <c r="J431" s="2" t="n"/>
+      <c r="K431" s="2" t="n"/>
+      <c r="L431" s="2" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n"/>
@@ -5759,6 +6649,8 @@
       <c r="H432" s="2" t="n"/>
       <c r="I432" s="2" t="n"/>
       <c r="J432" s="2" t="n"/>
+      <c r="K432" s="2" t="n"/>
+      <c r="L432" s="2" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n"/>
@@ -5771,6 +6663,8 @@
       <c r="H433" s="2" t="n"/>
       <c r="I433" s="2" t="n"/>
       <c r="J433" s="2" t="n"/>
+      <c r="K433" s="2" t="n"/>
+      <c r="L433" s="2" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n"/>
@@ -5783,6 +6677,8 @@
       <c r="H434" s="2" t="n"/>
       <c r="I434" s="2" t="n"/>
       <c r="J434" s="2" t="n"/>
+      <c r="K434" s="2" t="n"/>
+      <c r="L434" s="2" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n"/>
@@ -5795,6 +6691,8 @@
       <c r="H435" s="2" t="n"/>
       <c r="I435" s="2" t="n"/>
       <c r="J435" s="2" t="n"/>
+      <c r="K435" s="2" t="n"/>
+      <c r="L435" s="2" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n"/>
@@ -5807,6 +6705,8 @@
       <c r="H436" s="2" t="n"/>
       <c r="I436" s="2" t="n"/>
       <c r="J436" s="2" t="n"/>
+      <c r="K436" s="2" t="n"/>
+      <c r="L436" s="2" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n"/>
@@ -5819,6 +6719,8 @@
       <c r="H437" s="2" t="n"/>
       <c r="I437" s="2" t="n"/>
       <c r="J437" s="2" t="n"/>
+      <c r="K437" s="2" t="n"/>
+      <c r="L437" s="2" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n"/>
@@ -5831,6 +6733,8 @@
       <c r="H438" s="2" t="n"/>
       <c r="I438" s="2" t="n"/>
       <c r="J438" s="2" t="n"/>
+      <c r="K438" s="2" t="n"/>
+      <c r="L438" s="2" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n"/>
@@ -5843,6 +6747,8 @@
       <c r="H439" s="2" t="n"/>
       <c r="I439" s="2" t="n"/>
       <c r="J439" s="2" t="n"/>
+      <c r="K439" s="2" t="n"/>
+      <c r="L439" s="2" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n"/>
@@ -5855,6 +6761,8 @@
       <c r="H440" s="2" t="n"/>
       <c r="I440" s="2" t="n"/>
       <c r="J440" s="2" t="n"/>
+      <c r="K440" s="2" t="n"/>
+      <c r="L440" s="2" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n"/>
@@ -5867,6 +6775,8 @@
       <c r="H441" s="2" t="n"/>
       <c r="I441" s="2" t="n"/>
       <c r="J441" s="2" t="n"/>
+      <c r="K441" s="2" t="n"/>
+      <c r="L441" s="2" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n"/>
@@ -5879,6 +6789,8 @@
       <c r="H442" s="2" t="n"/>
       <c r="I442" s="2" t="n"/>
       <c r="J442" s="2" t="n"/>
+      <c r="K442" s="2" t="n"/>
+      <c r="L442" s="2" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n"/>
@@ -5891,6 +6803,8 @@
       <c r="H443" s="2" t="n"/>
       <c r="I443" s="2" t="n"/>
       <c r="J443" s="2" t="n"/>
+      <c r="K443" s="2" t="n"/>
+      <c r="L443" s="2" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n"/>
@@ -5903,6 +6817,8 @@
       <c r="H444" s="2" t="n"/>
       <c r="I444" s="2" t="n"/>
       <c r="J444" s="2" t="n"/>
+      <c r="K444" s="2" t="n"/>
+      <c r="L444" s="2" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n"/>
@@ -5915,6 +6831,8 @@
       <c r="H445" s="2" t="n"/>
       <c r="I445" s="2" t="n"/>
       <c r="J445" s="2" t="n"/>
+      <c r="K445" s="2" t="n"/>
+      <c r="L445" s="2" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n"/>
@@ -5927,6 +6845,8 @@
       <c r="H446" s="2" t="n"/>
       <c r="I446" s="2" t="n"/>
       <c r="J446" s="2" t="n"/>
+      <c r="K446" s="2" t="n"/>
+      <c r="L446" s="2" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n"/>
@@ -5939,6 +6859,8 @@
       <c r="H447" s="2" t="n"/>
       <c r="I447" s="2" t="n"/>
       <c r="J447" s="2" t="n"/>
+      <c r="K447" s="2" t="n"/>
+      <c r="L447" s="2" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n"/>
@@ -5951,6 +6873,8 @@
       <c r="H448" s="2" t="n"/>
       <c r="I448" s="2" t="n"/>
       <c r="J448" s="2" t="n"/>
+      <c r="K448" s="2" t="n"/>
+      <c r="L448" s="2" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n"/>
@@ -5963,6 +6887,8 @@
       <c r="H449" s="2" t="n"/>
       <c r="I449" s="2" t="n"/>
       <c r="J449" s="2" t="n"/>
+      <c r="K449" s="2" t="n"/>
+      <c r="L449" s="2" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n"/>
@@ -5975,6 +6901,8 @@
       <c r="H450" s="2" t="n"/>
       <c r="I450" s="2" t="n"/>
       <c r="J450" s="2" t="n"/>
+      <c r="K450" s="2" t="n"/>
+      <c r="L450" s="2" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n"/>
@@ -5987,6 +6915,8 @@
       <c r="H451" s="2" t="n"/>
       <c r="I451" s="2" t="n"/>
       <c r="J451" s="2" t="n"/>
+      <c r="K451" s="2" t="n"/>
+      <c r="L451" s="2" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n"/>
@@ -5999,6 +6929,8 @@
       <c r="H452" s="2" t="n"/>
       <c r="I452" s="2" t="n"/>
       <c r="J452" s="2" t="n"/>
+      <c r="K452" s="2" t="n"/>
+      <c r="L452" s="2" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n"/>
@@ -6011,6 +6943,8 @@
       <c r="H453" s="2" t="n"/>
       <c r="I453" s="2" t="n"/>
       <c r="J453" s="2" t="n"/>
+      <c r="K453" s="2" t="n"/>
+      <c r="L453" s="2" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n"/>
@@ -6023,6 +6957,8 @@
       <c r="H454" s="2" t="n"/>
       <c r="I454" s="2" t="n"/>
       <c r="J454" s="2" t="n"/>
+      <c r="K454" s="2" t="n"/>
+      <c r="L454" s="2" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n"/>
@@ -6035,6 +6971,8 @@
       <c r="H455" s="2" t="n"/>
       <c r="I455" s="2" t="n"/>
       <c r="J455" s="2" t="n"/>
+      <c r="K455" s="2" t="n"/>
+      <c r="L455" s="2" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n"/>
@@ -6047,6 +6985,8 @@
       <c r="H456" s="2" t="n"/>
       <c r="I456" s="2" t="n"/>
       <c r="J456" s="2" t="n"/>
+      <c r="K456" s="2" t="n"/>
+      <c r="L456" s="2" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n"/>
@@ -6059,6 +6999,8 @@
       <c r="H457" s="2" t="n"/>
       <c r="I457" s="2" t="n"/>
       <c r="J457" s="2" t="n"/>
+      <c r="K457" s="2" t="n"/>
+      <c r="L457" s="2" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n"/>
@@ -6071,6 +7013,8 @@
       <c r="H458" s="2" t="n"/>
       <c r="I458" s="2" t="n"/>
       <c r="J458" s="2" t="n"/>
+      <c r="K458" s="2" t="n"/>
+      <c r="L458" s="2" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n"/>
@@ -6083,6 +7027,8 @@
       <c r="H459" s="2" t="n"/>
       <c r="I459" s="2" t="n"/>
       <c r="J459" s="2" t="n"/>
+      <c r="K459" s="2" t="n"/>
+      <c r="L459" s="2" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n"/>
@@ -6095,6 +7041,8 @@
       <c r="H460" s="2" t="n"/>
       <c r="I460" s="2" t="n"/>
       <c r="J460" s="2" t="n"/>
+      <c r="K460" s="2" t="n"/>
+      <c r="L460" s="2" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n"/>
@@ -6107,6 +7055,8 @@
       <c r="H461" s="2" t="n"/>
       <c r="I461" s="2" t="n"/>
       <c r="J461" s="2" t="n"/>
+      <c r="K461" s="2" t="n"/>
+      <c r="L461" s="2" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n"/>
@@ -6119,6 +7069,8 @@
       <c r="H462" s="2" t="n"/>
       <c r="I462" s="2" t="n"/>
       <c r="J462" s="2" t="n"/>
+      <c r="K462" s="2" t="n"/>
+      <c r="L462" s="2" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n"/>
@@ -6131,6 +7083,8 @@
       <c r="H463" s="2" t="n"/>
       <c r="I463" s="2" t="n"/>
       <c r="J463" s="2" t="n"/>
+      <c r="K463" s="2" t="n"/>
+      <c r="L463" s="2" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n"/>
@@ -6143,6 +7097,8 @@
       <c r="H464" s="2" t="n"/>
       <c r="I464" s="2" t="n"/>
       <c r="J464" s="2" t="n"/>
+      <c r="K464" s="2" t="n"/>
+      <c r="L464" s="2" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n"/>
@@ -6155,6 +7111,8 @@
       <c r="H465" s="2" t="n"/>
       <c r="I465" s="2" t="n"/>
       <c r="J465" s="2" t="n"/>
+      <c r="K465" s="2" t="n"/>
+      <c r="L465" s="2" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n"/>
@@ -6167,6 +7125,8 @@
       <c r="H466" s="2" t="n"/>
       <c r="I466" s="2" t="n"/>
       <c r="J466" s="2" t="n"/>
+      <c r="K466" s="2" t="n"/>
+      <c r="L466" s="2" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n"/>
@@ -6179,6 +7139,8 @@
       <c r="H467" s="2" t="n"/>
       <c r="I467" s="2" t="n"/>
       <c r="J467" s="2" t="n"/>
+      <c r="K467" s="2" t="n"/>
+      <c r="L467" s="2" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n"/>
@@ -6191,6 +7153,8 @@
       <c r="H468" s="2" t="n"/>
       <c r="I468" s="2" t="n"/>
       <c r="J468" s="2" t="n"/>
+      <c r="K468" s="2" t="n"/>
+      <c r="L468" s="2" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n"/>
@@ -6203,6 +7167,8 @@
       <c r="H469" s="2" t="n"/>
       <c r="I469" s="2" t="n"/>
       <c r="J469" s="2" t="n"/>
+      <c r="K469" s="2" t="n"/>
+      <c r="L469" s="2" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n"/>
@@ -6215,6 +7181,8 @@
       <c r="H470" s="2" t="n"/>
       <c r="I470" s="2" t="n"/>
       <c r="J470" s="2" t="n"/>
+      <c r="K470" s="2" t="n"/>
+      <c r="L470" s="2" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n"/>
@@ -6227,6 +7195,8 @@
       <c r="H471" s="2" t="n"/>
       <c r="I471" s="2" t="n"/>
       <c r="J471" s="2" t="n"/>
+      <c r="K471" s="2" t="n"/>
+      <c r="L471" s="2" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n"/>
@@ -6239,6 +7209,8 @@
       <c r="H472" s="2" t="n"/>
       <c r="I472" s="2" t="n"/>
       <c r="J472" s="2" t="n"/>
+      <c r="K472" s="2" t="n"/>
+      <c r="L472" s="2" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n"/>
@@ -6251,6 +7223,8 @@
       <c r="H473" s="2" t="n"/>
       <c r="I473" s="2" t="n"/>
       <c r="J473" s="2" t="n"/>
+      <c r="K473" s="2" t="n"/>
+      <c r="L473" s="2" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n"/>
@@ -6263,6 +7237,8 @@
       <c r="H474" s="2" t="n"/>
       <c r="I474" s="2" t="n"/>
       <c r="J474" s="2" t="n"/>
+      <c r="K474" s="2" t="n"/>
+      <c r="L474" s="2" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n"/>
@@ -6275,6 +7251,8 @@
       <c r="H475" s="2" t="n"/>
       <c r="I475" s="2" t="n"/>
       <c r="J475" s="2" t="n"/>
+      <c r="K475" s="2" t="n"/>
+      <c r="L475" s="2" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n"/>
@@ -6287,6 +7265,8 @@
       <c r="H476" s="2" t="n"/>
       <c r="I476" s="2" t="n"/>
       <c r="J476" s="2" t="n"/>
+      <c r="K476" s="2" t="n"/>
+      <c r="L476" s="2" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n"/>
@@ -6299,6 +7279,8 @@
       <c r="H477" s="2" t="n"/>
       <c r="I477" s="2" t="n"/>
       <c r="J477" s="2" t="n"/>
+      <c r="K477" s="2" t="n"/>
+      <c r="L477" s="2" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n"/>
@@ -6311,6 +7293,8 @@
       <c r="H478" s="2" t="n"/>
       <c r="I478" s="2" t="n"/>
       <c r="J478" s="2" t="n"/>
+      <c r="K478" s="2" t="n"/>
+      <c r="L478" s="2" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n"/>
@@ -6323,6 +7307,8 @@
       <c r="H479" s="2" t="n"/>
       <c r="I479" s="2" t="n"/>
       <c r="J479" s="2" t="n"/>
+      <c r="K479" s="2" t="n"/>
+      <c r="L479" s="2" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n"/>
@@ -6335,6 +7321,8 @@
       <c r="H480" s="2" t="n"/>
       <c r="I480" s="2" t="n"/>
       <c r="J480" s="2" t="n"/>
+      <c r="K480" s="2" t="n"/>
+      <c r="L480" s="2" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n"/>
@@ -6347,6 +7335,8 @@
       <c r="H481" s="2" t="n"/>
       <c r="I481" s="2" t="n"/>
       <c r="J481" s="2" t="n"/>
+      <c r="K481" s="2" t="n"/>
+      <c r="L481" s="2" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="2" t="n"/>
@@ -6359,6 +7349,8 @@
       <c r="H482" s="2" t="n"/>
       <c r="I482" s="2" t="n"/>
       <c r="J482" s="2" t="n"/>
+      <c r="K482" s="2" t="n"/>
+      <c r="L482" s="2" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="2" t="n"/>
@@ -6371,6 +7363,8 @@
       <c r="H483" s="2" t="n"/>
       <c r="I483" s="2" t="n"/>
       <c r="J483" s="2" t="n"/>
+      <c r="K483" s="2" t="n"/>
+      <c r="L483" s="2" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="2" t="n"/>
@@ -6383,6 +7377,8 @@
       <c r="H484" s="2" t="n"/>
       <c r="I484" s="2" t="n"/>
       <c r="J484" s="2" t="n"/>
+      <c r="K484" s="2" t="n"/>
+      <c r="L484" s="2" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="2" t="n"/>
@@ -6395,6 +7391,8 @@
       <c r="H485" s="2" t="n"/>
       <c r="I485" s="2" t="n"/>
       <c r="J485" s="2" t="n"/>
+      <c r="K485" s="2" t="n"/>
+      <c r="L485" s="2" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="2" t="n"/>
@@ -6407,6 +7405,8 @@
       <c r="H486" s="2" t="n"/>
       <c r="I486" s="2" t="n"/>
       <c r="J486" s="2" t="n"/>
+      <c r="K486" s="2" t="n"/>
+      <c r="L486" s="2" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="2" t="n"/>
@@ -6419,6 +7419,8 @@
       <c r="H487" s="2" t="n"/>
       <c r="I487" s="2" t="n"/>
       <c r="J487" s="2" t="n"/>
+      <c r="K487" s="2" t="n"/>
+      <c r="L487" s="2" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="2" t="n"/>
@@ -6431,6 +7433,8 @@
       <c r="H488" s="2" t="n"/>
       <c r="I488" s="2" t="n"/>
       <c r="J488" s="2" t="n"/>
+      <c r="K488" s="2" t="n"/>
+      <c r="L488" s="2" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n"/>
@@ -6443,6 +7447,8 @@
       <c r="H489" s="2" t="n"/>
       <c r="I489" s="2" t="n"/>
       <c r="J489" s="2" t="n"/>
+      <c r="K489" s="2" t="n"/>
+      <c r="L489" s="2" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n"/>
@@ -6455,6 +7461,8 @@
       <c r="H490" s="2" t="n"/>
       <c r="I490" s="2" t="n"/>
       <c r="J490" s="2" t="n"/>
+      <c r="K490" s="2" t="n"/>
+      <c r="L490" s="2" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n"/>
@@ -6467,6 +7475,8 @@
       <c r="H491" s="2" t="n"/>
       <c r="I491" s="2" t="n"/>
       <c r="J491" s="2" t="n"/>
+      <c r="K491" s="2" t="n"/>
+      <c r="L491" s="2" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n"/>
@@ -6479,6 +7489,8 @@
       <c r="H492" s="2" t="n"/>
       <c r="I492" s="2" t="n"/>
       <c r="J492" s="2" t="n"/>
+      <c r="K492" s="2" t="n"/>
+      <c r="L492" s="2" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n"/>
@@ -6491,6 +7503,8 @@
       <c r="H493" s="2" t="n"/>
       <c r="I493" s="2" t="n"/>
       <c r="J493" s="2" t="n"/>
+      <c r="K493" s="2" t="n"/>
+      <c r="L493" s="2" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="2" t="n"/>
@@ -6503,6 +7517,8 @@
       <c r="H494" s="2" t="n"/>
       <c r="I494" s="2" t="n"/>
       <c r="J494" s="2" t="n"/>
+      <c r="K494" s="2" t="n"/>
+      <c r="L494" s="2" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="2" t="n"/>
@@ -6515,6 +7531,8 @@
       <c r="H495" s="2" t="n"/>
       <c r="I495" s="2" t="n"/>
       <c r="J495" s="2" t="n"/>
+      <c r="K495" s="2" t="n"/>
+      <c r="L495" s="2" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="n"/>
@@ -6527,6 +7545,8 @@
       <c r="H496" s="2" t="n"/>
       <c r="I496" s="2" t="n"/>
       <c r="J496" s="2" t="n"/>
+      <c r="K496" s="2" t="n"/>
+      <c r="L496" s="2" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="2" t="n"/>
@@ -6539,6 +7559,8 @@
       <c r="H497" s="2" t="n"/>
       <c r="I497" s="2" t="n"/>
       <c r="J497" s="2" t="n"/>
+      <c r="K497" s="2" t="n"/>
+      <c r="L497" s="2" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="2" t="n"/>
@@ -6551,6 +7573,8 @@
       <c r="H498" s="2" t="n"/>
       <c r="I498" s="2" t="n"/>
       <c r="J498" s="2" t="n"/>
+      <c r="K498" s="2" t="n"/>
+      <c r="L498" s="2" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="2" t="n"/>
@@ -6563,6 +7587,8 @@
       <c r="H499" s="2" t="n"/>
       <c r="I499" s="2" t="n"/>
       <c r="J499" s="2" t="n"/>
+      <c r="K499" s="2" t="n"/>
+      <c r="L499" s="2" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="2" t="n"/>
@@ -6575,11 +7601,19 @@
       <c r="H500" s="2" t="n"/>
       <c r="I500" s="2" t="n"/>
       <c r="J500" s="2" t="n"/>
+      <c r="K500" s="2" t="n"/>
+      <c r="L500" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Distrito inválido" error="Selecciona un distrito de la lista." type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Distrito inválido" error="Seleccione un valor de la lista." type="list">
       <formula1>=ListaDistritos</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Tipo de activo inválido" error="Seleccione un valor de la lista." type="list">
+      <formula1>"Poste MT,Suministro,Subestación"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Criticidad inválida" error="Seleccione un valor de la lista." type="list">
+      <formula1>"Riesgo Inminente,Tipo A,Tipo B,Tipo C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>